<commit_message>
Added figures of gold prices
</commit_message>
<xml_diff>
--- a/Module 2/Week 6 - Diversification and portfolio optimization/Homework 1 example.xlsx
+++ b/Module 2/Week 6 - Diversification and portfolio optimization/Homework 1 example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Risk-free" sheetId="1" state="visible" r:id="rId3"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="45">
   <si>
     <t xml:space="preserve">Month</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t xml:space="preserve">Vol of excess return:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sharpe ratio:</t>
   </si>
   <si>
     <t xml:space="preserve">Correlation:</t>
@@ -120,9 +123,6 @@
   </si>
   <si>
     <t xml:space="preserve">Scaled weights:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sharpe ratio:</t>
   </si>
   <si>
     <t xml:space="preserve">2. Find the optimal allocation between risk-free saving, and the risky portfolio above, for a given investor</t>
@@ -181,7 +181,7 @@
     <numFmt numFmtId="170" formatCode="0.000000"/>
     <numFmt numFmtId="171" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -221,13 +221,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -240,12 +235,6 @@
     </font>
     <font>
       <sz val="13"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -315,7 +304,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -360,14 +349,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -376,15 +357,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -416,7 +401,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -424,11 +409,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -555,6 +536,9 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
@@ -574,6 +558,9 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
@@ -637,11 +624,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="29240909"/>
-        <c:axId val="26773768"/>
+        <c:axId val="24924299"/>
+        <c:axId val="98336103"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="29240909"/>
+        <c:axId val="24924299"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -664,17 +651,20 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26773768"/>
+        <c:crossAx val="98336103"/>
         <c:crossesAt val="0"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="26773768"/>
+        <c:axId val="98336103"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -706,14 +696,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29240909"/>
+        <c:crossAx val="24924299"/>
         <c:crossesAt val="0"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -787,7 +780,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Just FBDIX and FKUTX'!$E$10:$E$10</c:f>
+              <c:f>'Just FBDIX and FKUTX'!$E$11:$E$11</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -844,7 +837,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'Just FBDIX and FKUTX'!$D$11:$D$62</c:f>
+              <c:f>'Just FBDIX and FKUTX'!$D$12:$D$63</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="52"/>
@@ -1009,7 +1002,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Just FBDIX and FKUTX'!$E$11:$E$62</c:f>
+              <c:f>'Just FBDIX and FKUTX'!$E$12:$E$63</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="52"/>
@@ -1174,11 +1167,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="56372322"/>
-        <c:axId val="13527316"/>
+        <c:axId val="78453890"/>
+        <c:axId val="92325829"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="56372322"/>
+        <c:axId val="78453890"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1243,12 +1236,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13527316"/>
+        <c:crossAx val="92325829"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="13527316"/>
+        <c:axId val="92325829"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1322,7 +1315,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56372322"/>
+        <c:crossAx val="78453890"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1398,7 +1391,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Just FBDIX and FKUTX'!$E$10:$E$10</c:f>
+              <c:f>'Just FBDIX and FKUTX'!$E$11:$E$11</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1455,7 +1448,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'Just FBDIX and FKUTX'!$D$11:$D$62</c:f>
+              <c:f>'Just FBDIX and FKUTX'!$D$12:$D$63</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="52"/>
@@ -1620,7 +1613,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Just FBDIX and FKUTX'!$E$11:$E$62</c:f>
+              <c:f>'Just FBDIX and FKUTX'!$E$12:$E$63</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="52"/>
@@ -1850,7 +1843,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Just FBDIX and FKUTX'!$D$68:$D$118</c:f>
+              <c:f>'Just FBDIX and FKUTX'!$D$69:$D$119</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="51"/>
@@ -2012,7 +2005,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Just FBDIX and FKUTX'!$E$68:$E$118</c:f>
+              <c:f>'Just FBDIX and FKUTX'!$E$69:$E$119</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="51"/>
@@ -2174,11 +2167,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="57444296"/>
-        <c:axId val="47310828"/>
+        <c:axId val="54172901"/>
+        <c:axId val="34831283"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="57444296"/>
+        <c:axId val="54172901"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2243,12 +2236,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47310828"/>
+        <c:crossAx val="34831283"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="47310828"/>
+        <c:axId val="34831283"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2322,7 +2315,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57444296"/>
+        <c:crossAx val="54172901"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2353,16 +2346,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>393120</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>73800</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>6480</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>44640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>462960</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>158760</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>76320</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>129240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2370,8 +2363,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="2831400" y="424440"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:off x="4883400" y="219960"/>
+        <a:ext cx="5759280" cy="3239280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2390,14 +2383,14 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>241920</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>26280</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>201240</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>86760</xdr:rowOff>
+      <xdr:colOff>200880</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>86040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2405,8 +2398,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7401600" y="1603800"/>
-        <a:ext cx="7274520" cy="4091400"/>
+        <a:off x="7401600" y="1778760"/>
+        <a:ext cx="7274160" cy="4091040"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2420,14 +2413,14 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>253440</xdr:colOff>
-      <xdr:row>35</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>29520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>213480</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>135720</xdr:rowOff>
+      <xdr:colOff>213120</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>135360</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2435,8 +2428,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7413120" y="6163560"/>
-        <a:ext cx="7275240" cy="4838400"/>
+        <a:off x="7413120" y="6338880"/>
+        <a:ext cx="7274880" cy="4838040"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4583,14 +4576,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="23.35"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
     </row>
@@ -4639,206 +4632,223 @@
         <v>0.0609764265511527</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>6</v>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="13" t="n">
+        <f aca="false">B3/B4</f>
+        <v>0.179973921337807</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <f aca="false">C3/C4</f>
+        <v>0.170352560129778</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <f aca="false">D3/D4</f>
+        <v>0.125525014454168</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="22" t="n">
-        <f aca="false" t="array" ref="B7:D9">MMULT( TRANSPOSE( 'Demeaned excess returns'!B3:D242) , 'Demeaned excess returns'!B3:D242) / 239</f>
-        <v>0.00187756766263439</v>
-      </c>
-      <c r="C7" s="22" t="n">
-        <v>0.000962563231504759</v>
-      </c>
-      <c r="D7" s="22" t="n">
-        <v>0.00156328800379659</v>
+      <c r="C7" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="22" t="n">
-        <v>0.000962563231504759</v>
-      </c>
-      <c r="C8" s="22" t="n">
-        <v>0.00154601681310119</v>
-      </c>
-      <c r="D8" s="22" t="n">
-        <v>0.000578833690489693</v>
+        <v>4</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <f aca="false" t="array" ref="B8:D10">MMULT( TRANSPOSE( 'Demeaned excess returns'!B3:D242) , 'Demeaned excess returns'!B3:D242) / 239</f>
+        <v>0.00187756766263439</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>0.00096256323150476</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>0.00156328800379659</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>0.00096256323150476</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>0.00154601681310119</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>0.000578833690489693</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B10" s="21" t="n">
         <v>0.00156328800379659</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C10" s="21" t="n">
         <v>0.000578833690489693</v>
       </c>
-      <c r="D9" s="22" t="n">
-        <v>0.00371812459494811</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
+      <c r="D10" s="21" t="n">
+        <v>0.00371812459494812</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="8" t="s">
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D14" s="8" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="22" t="n">
-        <f aca="false" t="array" ref="B14:D14">TRANSPOSE( MMULT( MINVERSE( B7:D9 ), TRANSPOSE( B3:D3 ) ))</f>
-        <v>2.15038905940216</v>
-      </c>
-      <c r="C14" s="22" t="n">
-        <v>2.71998855366219</v>
-      </c>
-      <c r="D14" s="22" t="n">
-        <v>0.731005194184472</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="1" t="n">
-        <f aca="false">B14/SUM($B14:$D14)</f>
+      <c r="B15" s="21" t="n">
+        <f aca="false" t="array" ref="B15:D15">TRANSPOSE( MMULT( MINVERSE( B8:D10 ), TRANSPOSE( B3:D3 ) ))</f>
+        <v>2.15038905940215</v>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>2.71998855366219</v>
+      </c>
+      <c r="D15" s="21" t="n">
+        <v>0.731005194184472</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <f aca="false">B15/SUM($B15:$D15)</f>
         <v>0.383903249143999</v>
       </c>
-      <c r="C15" s="1" t="n">
-        <f aca="false">C14/SUM($B14:$D14)</f>
+      <c r="C16" s="1" t="n">
+        <f aca="false">C15/SUM($B15:$D15)</f>
         <v>0.485592334475376</v>
       </c>
-      <c r="D15" s="1" t="n">
-        <f aca="false">D14/SUM($B14:$D14)</f>
+      <c r="D16" s="1" t="n">
+        <f aca="false">D15/SUM($B15:$D15)</f>
         <v>0.130504416380625</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B17" s="10" t="n">
-        <f aca="false" t="array" ref="B17:B17">MMULT( B15:D15 , TRANSPOSE(B3:D3) )</f>
-        <v>0.00724531056504633</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" s="10" t="n">
-        <f aca="false" t="array" ref="B18:B18">SQRT( MMULT( B15:D15 , MMULT(B7:D9 , TRANSPOSE(B15:D15) ) ) )</f>
-        <v>0.0359650671861637</v>
+        <f aca="false" t="array" ref="B18:B18">MMULT( B16:D16 , TRANSPOSE(B3:D3) )</f>
+        <v>0.00724531056504632</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="22" t="n">
-        <f aca="false">B17/B18</f>
+        <v>13</v>
+      </c>
+      <c r="B19" s="10" t="n">
+        <f aca="false" t="array" ref="B19:B19">SQRT( MMULT( B16:D16 , MMULT(B8:D10 , TRANSPOSE(B16:D16) ) ) )</f>
+        <v>0.0359650671861637</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <f aca="false">B18/B19</f>
         <v>0.201454108998126</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B23" s="8" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="10" t="n">
-        <f aca="false">B17/(B23*B18^2)</f>
+      <c r="B25" s="10" t="n">
+        <f aca="false">B18/(B24*B19^2)</f>
         <v>0.700172850906102</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25" t="s">
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="24" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25"/>
-    </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
-        <v>37</v>
-      </c>
+      <c r="A28" s="24"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B29" s="10" t="n">
-        <f aca="false">1-B24</f>
-        <v>0.299827149093898</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B30" s="10" t="n">
-        <f aca="false">B24*B15</f>
-        <v>0.26879863242527</v>
+        <f aca="false">1-B25</f>
+        <v>0.299827149093898</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B31" s="10" t="n">
-        <f aca="false">B24*C15</f>
-        <v>0.339998569207774</v>
+        <f aca="false">B25*B16</f>
+        <v>0.268798632425269</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="10" t="n">
+        <f aca="false">B25*C16</f>
+        <v>0.339998569207774</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B32" s="10" t="n">
-        <f aca="false">B24*D15</f>
+      <c r="B33" s="10" t="n">
+        <f aca="false">B25*D16</f>
         <v>0.091375649273059</v>
       </c>
     </row>
@@ -4882,7 +4892,7 @@
       <c r="A2" s="4" t="n">
         <v>38322</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="25" t="s">
         <v>44</v>
       </c>
     </row>
@@ -25284,64 +25294,64 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="0" t="n">
+      <c r="B4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="10" t="n">
         <f aca="false">STDEV('Excess returns'!B3:B242)</f>
         <v>0.0433309088600088</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="1" t="n">
         <f aca="false">AVERAGE('Excess returns'!B3:B242)</f>
         <v>0.00779843358266689</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="10" t="n">
         <f aca="false">STDEV('Excess returns'!C3:C242)</f>
         <v>0.039319420304745</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="10" t="n">
         <f aca="false">AVERAGE('Excess returns'!C3:C242)</f>
         <v>0.00669816391173209</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <f aca="false">STDEV('Excess returns'!D3:D242)</f>
         <v>0.0609764265511527</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="10" t="n">
         <f aca="false">AVERAGE('Excess returns'!D3:D242)</f>
         <v>0.00765406682419694</v>
       </c>
@@ -25363,7 +25373,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="18.2"/>
@@ -25371,11 +25381,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="8" width="12.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="13" width="11.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="11" width="11.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
     </row>
@@ -25399,6 +25409,7 @@
         <f aca="false">AVERAGE('Excess returns'!D3:D242)</f>
         <v>0.00765406682419694</v>
       </c>
+      <c r="D3" s="13"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
@@ -25412,2540 +25423,2555 @@
         <f aca="false">STDEV('Excess returns'!D3:D242)</f>
         <v>0.0609764265511527</v>
       </c>
+      <c r="D4" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="15" t="n">
-        <f aca="false">CORREL('Excess returns'!C3:C242,'Excess returns'!D3:D242)</f>
-        <v>0.241426381441205</v>
-      </c>
+      <c r="B5" s="13" t="n">
+        <f aca="false">B3/B4</f>
+        <v>0.170352560129778</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <f aca="false">C3/C4</f>
+        <v>0.125525014454168</v>
+      </c>
+      <c r="D5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="15" t="n">
-        <f aca="false">B5*B4*C4</f>
+      <c r="B6" s="14" t="n">
+        <f aca="false">CORREL('Excess returns'!C3:C242,'Excess returns'!D3:D242)</f>
+        <v>0.241426381441205</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="14" t="n">
+        <f aca="false">B6*B4*C4</f>
         <v>0.000578833690489693</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
-        <v>16</v>
-      </c>
-    </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14"/>
+      <c r="A9" s="12" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="8" t="s">
+      <c r="A10" s="12"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="C11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E11" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="16" t="n">
-        <f aca="false">1-B11</f>
+      <c r="F11" s="16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <f aca="false">1-B12</f>
         <v>1</v>
       </c>
-      <c r="D11" s="10" t="n">
-        <f aca="false">SQRT( B11^2*B$4^2 + C11^2*C$4^2 + 2*B11*C11*B$6)</f>
+      <c r="D12" s="10" t="n">
+        <f aca="false">SQRT( B12^2*B$4^2 + C12^2*C$4^2 + 2*B12*C12*B$7)</f>
         <v>0.0609764265511527</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <f aca="false">B11*B$3 + C11*C$3</f>
-        <v>0.00765406682419694</v>
-      </c>
-      <c r="F11" s="18" t="n">
-        <f aca="false">E11/D11</f>
-        <v>0.125525014454168</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="1" t="n">
-        <f aca="false">B11+0.02</f>
-        <v>0.02</v>
-      </c>
-      <c r="C12" s="16" t="n">
-        <f aca="false">1-B12</f>
-        <v>0.98</v>
-      </c>
-      <c r="D12" s="10" t="n">
-        <f aca="false">SQRT( B12^2*B$4^2 + C12^2*C$4^2 + 2*B12*C12*B$6)</f>
-        <v>0.0599516100566165</v>
       </c>
       <c r="E12" s="10" t="n">
         <f aca="false">B12*B$3 + C12*C$3</f>
-        <v>0.00763494876594765</v>
-      </c>
-      <c r="F12" s="18" t="n">
+        <v>0.00765406682419694</v>
+      </c>
+      <c r="F12" s="17" t="n">
         <f aca="false">E12/D12</f>
-        <v>0.127351855250216</v>
+        <v>0.125525014454168</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="1" t="n">
         <f aca="false">B12+0.02</f>
-        <v>0.04</v>
-      </c>
-      <c r="C13" s="16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C13" s="15" t="n">
         <f aca="false">1-B13</f>
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">SQRT( B13^2*B$4^2 + C13^2*C$4^2 + 2*B13*C13*B$6)</f>
-        <v>0.0589368448513725</v>
+        <f aca="false">SQRT( B13^2*B$4^2 + C13^2*C$4^2 + 2*B13*C13*B$7)</f>
+        <v>0.0599516100566165</v>
       </c>
       <c r="E13" s="10" t="n">
         <f aca="false">B13*B$3 + C13*C$3</f>
-        <v>0.00761583070769835</v>
-      </c>
-      <c r="F13" s="18" t="n">
+        <v>0.00763494876594765</v>
+      </c>
+      <c r="F13" s="17" t="n">
         <f aca="false">E13/D13</f>
-        <v>0.129220197092397</v>
+        <v>0.127351855250216</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="1" t="n">
         <f aca="false">B13+0.02</f>
-        <v>0.06</v>
-      </c>
-      <c r="C14" s="16" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C14" s="15" t="n">
         <f aca="false">1-B14</f>
-        <v>0.94</v>
+        <v>0.96</v>
       </c>
       <c r="D14" s="10" t="n">
-        <f aca="false">SQRT( B14^2*B$4^2 + C14^2*C$4^2 + 2*B14*C14*B$6)</f>
-        <v>0.0579326591216954</v>
+        <f aca="false">SQRT( B14^2*B$4^2 + C14^2*C$4^2 + 2*B14*C14*B$7)</f>
+        <v>0.0589368448513725</v>
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">B14*B$3 + C14*C$3</f>
-        <v>0.00759671264944905</v>
-      </c>
-      <c r="F14" s="18" t="n">
+        <v>0.00761583070769835</v>
+      </c>
+      <c r="F14" s="17" t="n">
         <f aca="false">E14/D14</f>
-        <v>0.131130052799598</v>
+        <v>0.129220197092397</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="1" t="n">
         <f aca="false">B14+0.02</f>
-        <v>0.08</v>
-      </c>
-      <c r="C15" s="16" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C15" s="15" t="n">
         <f aca="false">1-B15</f>
-        <v>0.92</v>
+        <v>0.94</v>
       </c>
       <c r="D15" s="10" t="n">
-        <f aca="false">SQRT( B15^2*B$4^2 + C15^2*C$4^2 + 2*B15*C15*B$6)</f>
-        <v>0.0569396126085172</v>
+        <f aca="false">SQRT( B15^2*B$4^2 + C15^2*C$4^2 + 2*B15*C15*B$7)</f>
+        <v>0.0579326591216954</v>
       </c>
       <c r="E15" s="10" t="n">
         <f aca="false">B15*B$3 + C15*C$3</f>
-        <v>0.00757759459119976</v>
-      </c>
-      <c r="F15" s="18" t="n">
+        <v>0.00759671264944905</v>
+      </c>
+      <c r="F15" s="17" t="n">
         <f aca="false">E15/D15</f>
-        <v>0.133081245973673</v>
+        <v>0.131130052799598</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="1" t="n">
         <f aca="false">B15+0.02</f>
-        <v>0.1</v>
-      </c>
-      <c r="C16" s="16" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C16" s="15" t="n">
         <f aca="false">1-B16</f>
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="D16" s="10" t="n">
-        <f aca="false">SQRT( B16^2*B$4^2 + C16^2*C$4^2 + 2*B16*C16*B$6)</f>
-        <v>0.0559582983508892</v>
+        <f aca="false">SQRT( B16^2*B$4^2 + C16^2*C$4^2 + 2*B16*C16*B$7)</f>
+        <v>0.0569396126085172</v>
       </c>
       <c r="E16" s="10" t="n">
         <f aca="false">B16*B$3 + C16*C$3</f>
-        <v>0.00755847653295046</v>
-      </c>
-      <c r="F16" s="18" t="n">
+        <v>0.00757759459119976</v>
+      </c>
+      <c r="F16" s="17" t="n">
         <f aca="false">E16/D16</f>
-        <v>0.135073380637036</v>
+        <v>0.133081245973673</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="n">
         <f aca="false">B16+0.02</f>
-        <v>0.12</v>
-      </c>
-      <c r="C17" s="16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C17" s="15" t="n">
         <f aca="false">1-B17</f>
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="D17" s="10" t="n">
-        <f aca="false">SQRT( B17^2*B$4^2 + C17^2*C$4^2 + 2*B17*C17*B$6)</f>
-        <v>0.054989344457521</v>
+        <f aca="false">SQRT( B17^2*B$4^2 + C17^2*C$4^2 + 2*B17*C17*B$7)</f>
+        <v>0.0559582983508892</v>
       </c>
       <c r="E17" s="10" t="n">
         <f aca="false">B17*B$3 + C17*C$3</f>
-        <v>0.00753935847470116</v>
-      </c>
-      <c r="F17" s="18" t="n">
+        <v>0.00755847653295046</v>
+      </c>
+      <c r="F17" s="17" t="n">
         <f aca="false">E17/D17</f>
-        <v>0.137105807481034</v>
+        <v>0.135073380637036</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="n">
         <f aca="false">B17+0.02</f>
-        <v>0.14</v>
-      </c>
-      <c r="C18" s="16" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C18" s="15" t="n">
         <f aca="false">1-B18</f>
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="D18" s="10" t="n">
-        <f aca="false">SQRT( B18^2*B$4^2 + C18^2*C$4^2 + 2*B18*C18*B$6)</f>
-        <v>0.0540334158889694</v>
+        <f aca="false">SQRT( B18^2*B$4^2 + C18^2*C$4^2 + 2*B18*C18*B$7)</f>
+        <v>0.054989344457521</v>
       </c>
       <c r="E18" s="10" t="n">
         <f aca="false">B18*B$3 + C18*C$3</f>
-        <v>0.00752024041645186</v>
-      </c>
-      <c r="F18" s="18" t="n">
+        <v>0.00753935847470116</v>
+      </c>
+      <c r="F18" s="17" t="n">
         <f aca="false">E18/D18</f>
-        <v>0.139177586549495</v>
+        <v>0.137105807481034</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="n">
         <f aca="false">B18+0.02</f>
-        <v>0.16</v>
-      </c>
-      <c r="C19" s="16" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C19" s="15" t="n">
         <f aca="false">1-B19</f>
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="D19" s="10" t="n">
-        <f aca="false">SQRT( B19^2*B$4^2 + C19^2*C$4^2 + 2*B19*C19*B$6)</f>
-        <v>0.0530912162284347</v>
+        <f aca="false">SQRT( B19^2*B$4^2 + C19^2*C$4^2 + 2*B19*C19*B$7)</f>
+        <v>0.0540334158889694</v>
       </c>
       <c r="E19" s="10" t="n">
         <f aca="false">B19*B$3 + C19*C$3</f>
-        <v>0.00750112235820257</v>
-      </c>
-      <c r="F19" s="18" t="n">
+        <v>0.00752024041645186</v>
+      </c>
+      <c r="F19" s="17" t="n">
         <f aca="false">E19/D19</f>
-        <v>0.141287446230797</v>
+        <v>0.139177586549495</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="n">
         <f aca="false">B19+0.02</f>
-        <v>0.18</v>
-      </c>
-      <c r="C20" s="16" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="C20" s="15" t="n">
         <f aca="false">1-B20</f>
-        <v>0.82</v>
+        <v>0.84</v>
       </c>
       <c r="D20" s="10" t="n">
-        <f aca="false">SQRT( B20^2*B$4^2 + C20^2*C$4^2 + 2*B20*C20*B$6)</f>
-        <v>0.0521634894137667</v>
+        <f aca="false">SQRT( B20^2*B$4^2 + C20^2*C$4^2 + 2*B20*C20*B$7)</f>
+        <v>0.0530912162284347</v>
       </c>
       <c r="E20" s="10" t="n">
         <f aca="false">B20*B$3 + C20*C$3</f>
-        <v>0.00748200429995327</v>
-      </c>
-      <c r="F20" s="18" t="n">
+        <v>0.00750112235820257</v>
+      </c>
+      <c r="F20" s="17" t="n">
         <f aca="false">E20/D20</f>
-        <v>0.143433738502522</v>
+        <v>0.141287446230797</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="1" t="n">
         <f aca="false">B20+0.02</f>
-        <v>0.2</v>
-      </c>
-      <c r="C21" s="16" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="C21" s="15" t="n">
         <f aca="false">1-B21</f>
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="D21" s="10" t="n">
-        <f aca="false">SQRT( B21^2*B$4^2 + C21^2*C$4^2 + 2*B21*C21*B$6)</f>
-        <v>0.051251021397115</v>
+        <f aca="false">SQRT( B21^2*B$4^2 + C21^2*C$4^2 + 2*B21*C21*B$7)</f>
+        <v>0.0521634894137667</v>
       </c>
       <c r="E21" s="10" t="n">
         <f aca="false">B21*B$3 + C21*C$3</f>
-        <v>0.00746288624170397</v>
-      </c>
-      <c r="F21" s="18" t="n">
+        <v>0.00748200429995327</v>
+      </c>
+      <c r="F21" s="17" t="n">
         <f aca="false">E21/D21</f>
-        <v>0.145614390469964</v>
+        <v>0.143433738502522</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="n">
         <f aca="false">B21+0.02</f>
-        <v>0.22</v>
-      </c>
-      <c r="C22" s="16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C22" s="15" t="n">
         <f aca="false">1-B22</f>
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="D22" s="10" t="n">
-        <f aca="false">SQRT( B22^2*B$4^2 + C22^2*C$4^2 + 2*B22*C22*B$6)</f>
-        <v>0.0503546416916712</v>
+        <f aca="false">SQRT( B22^2*B$4^2 + C22^2*C$4^2 + 2*B22*C22*B$7)</f>
+        <v>0.051251021397115</v>
       </c>
       <c r="E22" s="10" t="n">
         <f aca="false">B22*B$3 + C22*C$3</f>
-        <v>0.00744376818345468</v>
-      </c>
-      <c r="F22" s="18" t="n">
+        <v>0.00746288624170397</v>
+      </c>
+      <c r="F22" s="17" t="n">
         <f aca="false">E22/D22</f>
-        <v>0.147826852369121</v>
+        <v>0.145614390469964</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="1" t="n">
         <f aca="false">B22+0.02</f>
-        <v>0.24</v>
-      </c>
-      <c r="C23" s="16" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C23" s="15" t="n">
         <f aca="false">1-B23</f>
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="D23" s="10" t="n">
-        <f aca="false">SQRT( B23^2*B$4^2 + C23^2*C$4^2 + 2*B23*C23*B$6)</f>
-        <v>0.0494752247571176</v>
+        <f aca="false">SQRT( B23^2*B$4^2 + C23^2*C$4^2 + 2*B23*C23*B$7)</f>
+        <v>0.0503546416916712</v>
       </c>
       <c r="E23" s="10" t="n">
         <f aca="false">B23*B$3 + C23*C$3</f>
-        <v>0.00742465012520538</v>
-      </c>
-      <c r="F23" s="18" t="n">
+        <v>0.00744376818345468</v>
+      </c>
+      <c r="F23" s="17" t="n">
         <f aca="false">E23/D23</f>
-        <v>0.150068042371799</v>
+        <v>0.147826852369121</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="1" t="n">
         <f aca="false">B23+0.02</f>
-        <v>0.26</v>
-      </c>
-      <c r="C24" s="16" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C24" s="15" t="n">
         <f aca="false">1-B24</f>
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="D24" s="10" t="n">
-        <f aca="false">SQRT( B24^2*B$4^2 + C24^2*C$4^2 + 2*B24*C24*B$6)</f>
-        <v>0.0486136911667862</v>
+        <f aca="false">SQRT( B24^2*B$4^2 + C24^2*C$4^2 + 2*B24*C24*B$7)</f>
+        <v>0.0494752247571176</v>
       </c>
       <c r="E24" s="10" t="n">
         <f aca="false">B24*B$3 + C24*C$3</f>
-        <v>0.00740553206695608</v>
-      </c>
-      <c r="F24" s="18" t="n">
+        <v>0.00742465012520538</v>
+      </c>
+      <c r="F24" s="17" t="n">
         <f aca="false">E24/D24</f>
-        <v>0.152334288740775</v>
+        <v>0.150068042371799</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="1" t="n">
         <f aca="false">B24+0.02</f>
-        <v>0.28</v>
-      </c>
-      <c r="C25" s="16" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="C25" s="15" t="n">
         <f aca="false">1-B25</f>
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="D25" s="10" t="n">
-        <f aca="false">SQRT( B25^2*B$4^2 + C25^2*C$4^2 + 2*B25*C25*B$6)</f>
-        <v>0.0477710084902306</v>
+        <f aca="false">SQRT( B25^2*B$4^2 + C25^2*C$4^2 + 2*B25*C25*B$7)</f>
+        <v>0.0486136911667862</v>
       </c>
       <c r="E25" s="10" t="n">
         <f aca="false">B25*B$3 + C25*C$3</f>
-        <v>0.00738641400870678</v>
-      </c>
-      <c r="F25" s="18" t="n">
+        <v>0.00740553206695608</v>
+      </c>
+      <c r="F25" s="17" t="n">
         <f aca="false">E25/D25</f>
-        <v>0.154621270141646</v>
+        <v>0.152334288740775</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="1" t="n">
         <f aca="false">B25+0.02</f>
-        <v>0.3</v>
-      </c>
-      <c r="C26" s="16" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C26" s="15" t="n">
         <f aca="false">1-B26</f>
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="D26" s="10" t="n">
-        <f aca="false">SQRT( B26^2*B$4^2 + C26^2*C$4^2 + 2*B26*C26*B$6)</f>
-        <v>0.0469481918151206</v>
+        <f aca="false">SQRT( B26^2*B$4^2 + C26^2*C$4^2 + 2*B26*C26*B$7)</f>
+        <v>0.0477710084902306</v>
       </c>
       <c r="E26" s="10" t="n">
         <f aca="false">B26*B$3 + C26*C$3</f>
-        <v>0.00736729595045749</v>
-      </c>
-      <c r="F26" s="18" t="n">
+        <v>0.00738641400870678</v>
+      </c>
+      <c r="F26" s="17" t="n">
         <f aca="false">E26/D26</f>
-        <v>0.156923955228553</v>
+        <v>0.154621270141646</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="1" t="n">
         <f aca="false">B26+0.02</f>
-        <v>0.32</v>
-      </c>
-      <c r="C27" s="16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C27" s="15" t="n">
         <f aca="false">1-B27</f>
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
       <c r="D27" s="10" t="n">
-        <f aca="false">SQRT( B27^2*B$4^2 + C27^2*C$4^2 + 2*B27*C27*B$6)</f>
-        <v>0.0461463038223722</v>
+        <f aca="false">SQRT( B27^2*B$4^2 + C27^2*C$4^2 + 2*B27*C27*B$7)</f>
+        <v>0.0469481918151206</v>
       </c>
       <c r="E27" s="10" t="n">
         <f aca="false">B27*B$3 + C27*C$3</f>
-        <v>0.00734817789220819</v>
-      </c>
-      <c r="F27" s="18" t="n">
+        <v>0.00736729595045749</v>
+      </c>
+      <c r="F27" s="17" t="n">
         <f aca="false">E27/D27</f>
-        <v>0.15923654298496</v>
+        <v>0.156923955228553</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="1" t="n">
         <f aca="false">B27+0.02</f>
-        <v>0.34</v>
-      </c>
-      <c r="C28" s="16" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="C28" s="15" t="n">
         <f aca="false">1-B28</f>
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="D28" s="10" t="n">
-        <f aca="false">SQRT( B28^2*B$4^2 + C28^2*C$4^2 + 2*B28*C28*B$6)</f>
-        <v>0.0453664543186446</v>
+        <f aca="false">SQRT( B28^2*B$4^2 + C28^2*C$4^2 + 2*B28*C28*B$7)</f>
+        <v>0.0461463038223722</v>
       </c>
       <c r="E28" s="10" t="n">
         <f aca="false">B28*B$3 + C28*C$3</f>
-        <v>0.00732905983395889</v>
-      </c>
-      <c r="F28" s="18" t="n">
+        <v>0.00734817789220819</v>
+      </c>
+      <c r="F28" s="17" t="n">
         <f aca="false">E28/D28</f>
-        <v>0.161552405715489</v>
+        <v>0.15923654298496</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="1" t="n">
         <f aca="false">B28+0.02</f>
-        <v>0.36</v>
-      </c>
-      <c r="C29" s="16" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="C29" s="15" t="n">
         <f aca="false">1-B29</f>
-        <v>0.64</v>
+        <v>0.66</v>
       </c>
       <c r="D29" s="10" t="n">
-        <f aca="false">SQRT( B29^2*B$4^2 + C29^2*C$4^2 + 2*B29*C29*B$6)</f>
-        <v>0.0446097991213401</v>
+        <f aca="false">SQRT( B29^2*B$4^2 + C29^2*C$4^2 + 2*B29*C29*B$7)</f>
+        <v>0.0453664543186446</v>
       </c>
       <c r="E29" s="10" t="n">
         <f aca="false">B29*B$3 + C29*C$3</f>
-        <v>0.0073099417757096</v>
-      </c>
-      <c r="F29" s="18" t="n">
+        <v>0.00732905983395889</v>
+      </c>
+      <c r="F29" s="17" t="n">
         <f aca="false">E29/D29</f>
-        <v>0.163864037043214</v>
+        <v>0.161552405715489</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="1" t="n">
         <f aca="false">B29+0.02</f>
-        <v>0.38</v>
-      </c>
-      <c r="C30" s="16" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C30" s="15" t="n">
         <f aca="false">1-B30</f>
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
       <c r="D30" s="10" t="n">
-        <f aca="false">SQRT( B30^2*B$4^2 + C30^2*C$4^2 + 2*B30*C30*B$6)</f>
-        <v>0.0438775381837747</v>
+        <f aca="false">SQRT( B30^2*B$4^2 + C30^2*C$4^2 + 2*B30*C30*B$7)</f>
+        <v>0.0446097991213401</v>
       </c>
       <c r="E30" s="10" t="n">
         <f aca="false">B30*B$3 + C30*C$3</f>
-        <v>0.0072908237174603</v>
-      </c>
-      <c r="F30" s="18" t="n">
+        <v>0.0073099417757096</v>
+      </c>
+      <c r="F30" s="17" t="n">
         <f aca="false">E30/D30</f>
-        <v>0.166163007754075</v>
+        <v>0.163864037043214</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="1" t="n">
         <f aca="false">B30+0.02</f>
-        <v>0.4</v>
-      </c>
-      <c r="C31" s="16" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="C31" s="15" t="n">
         <f aca="false">1-B31</f>
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="D31" s="10" t="n">
-        <f aca="false">SQRT( B31^2*B$4^2 + C31^2*C$4^2 + 2*B31*C31*B$6)</f>
-        <v>0.0431709128431698</v>
+        <f aca="false">SQRT( B31^2*B$4^2 + C31^2*C$4^2 + 2*B31*C31*B$7)</f>
+        <v>0.0438775381837747</v>
       </c>
       <c r="E31" s="10" t="n">
         <f aca="false">B31*B$3 + C31*C$3</f>
-        <v>0.007271705659211</v>
-      </c>
-      <c r="F31" s="18" t="n">
+        <v>0.0072908237174603</v>
+      </c>
+      <c r="F31" s="17" t="n">
         <f aca="false">E31/D31</f>
-        <v>0.168439932822997</v>
+        <v>0.166163007754075</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="1" t="n">
         <f aca="false">B31+0.02</f>
-        <v>0.42</v>
-      </c>
-      <c r="C32" s="16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C32" s="15" t="n">
         <f aca="false">1-B32</f>
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="D32" s="10" t="n">
-        <f aca="false">SQRT( B32^2*B$4^2 + C32^2*C$4^2 + 2*B32*C32*B$6)</f>
-        <v>0.0424912020726429</v>
+        <f aca="false">SQRT( B32^2*B$4^2 + C32^2*C$4^2 + 2*B32*C32*B$7)</f>
+        <v>0.0431709128431698</v>
       </c>
       <c r="E32" s="10" t="n">
         <f aca="false">B32*B$3 + C32*C$3</f>
-        <v>0.00725258760096171</v>
-      </c>
-      <c r="F32" s="18" t="n">
+        <v>0.007271705659211</v>
+      </c>
+      <c r="F32" s="17" t="n">
         <f aca="false">E32/D32</f>
-        <v>0.170684453420797</v>
+        <v>0.168439932822997</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="1" t="n">
         <f aca="false">B32+0.02</f>
-        <v>0.44</v>
-      </c>
-      <c r="C33" s="16" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="C33" s="15" t="n">
         <f aca="false">1-B33</f>
-        <v>0.56</v>
+        <v>0.58</v>
       </c>
       <c r="D33" s="10" t="n">
-        <f aca="false">SQRT( B33^2*B$4^2 + C33^2*C$4^2 + 2*B33*C33*B$6)</f>
-        <v>0.0418397176217221</v>
+        <f aca="false">SQRT( B33^2*B$4^2 + C33^2*C$4^2 + 2*B33*C33*B$7)</f>
+        <v>0.0424912020726429</v>
       </c>
       <c r="E33" s="10" t="n">
         <f aca="false">B33*B$3 + C33*C$3</f>
-        <v>0.00723346954271241</v>
-      </c>
-      <c r="F33" s="18" t="n">
+        <v>0.00725258760096171</v>
+      </c>
+      <c r="F33" s="17" t="n">
         <f aca="false">E33/D33</f>
-        <v>0.172885238091497</v>
+        <v>0.170684453420797</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="1" t="n">
         <f aca="false">B33+0.02</f>
-        <v>0.46</v>
-      </c>
-      <c r="C34" s="16" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="C34" s="15" t="n">
         <f aca="false">1-B34</f>
-        <v>0.54</v>
+        <v>0.56</v>
       </c>
       <c r="D34" s="10" t="n">
-        <f aca="false">SQRT( B34^2*B$4^2 + C34^2*C$4^2 + 2*B34*C34*B$6)</f>
-        <v>0.041217797939414</v>
+        <f aca="false">SQRT( B34^2*B$4^2 + C34^2*C$4^2 + 2*B34*C34*B$7)</f>
+        <v>0.0418397176217221</v>
       </c>
       <c r="E34" s="10" t="n">
         <f aca="false">B34*B$3 + C34*C$3</f>
-        <v>0.00721435148446311</v>
-      </c>
-      <c r="F34" s="18" t="n">
+        <v>0.00723346954271241</v>
+      </c>
+      <c r="F34" s="17" t="n">
         <f aca="false">E34/D34</f>
-        <v>0.175030007548377</v>
+        <v>0.172885238091497</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="1" t="n">
         <f aca="false">B34+0.02</f>
-        <v>0.48</v>
-      </c>
-      <c r="C35" s="16" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="C35" s="15" t="n">
         <f aca="false">1-B35</f>
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="D35" s="10" t="n">
-        <f aca="false">SQRT( B35^2*B$4^2 + C35^2*C$4^2 + 2*B35*C35*B$6)</f>
-        <v>0.040626800790918</v>
+        <f aca="false">SQRT( B35^2*B$4^2 + C35^2*C$4^2 + 2*B35*C35*B$7)</f>
+        <v>0.041217797939414</v>
       </c>
       <c r="E35" s="10" t="n">
         <f aca="false">B35*B$3 + C35*C$3</f>
-        <v>0.00719523342621381</v>
-      </c>
-      <c r="F35" s="18" t="n">
+        <v>0.00721435148446311</v>
+      </c>
+      <c r="F35" s="17" t="n">
         <f aca="false">E35/D35</f>
-        <v>0.177105587595819</v>
+        <v>0.175030007548377</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="1" t="n">
         <f aca="false">B35+0.02</f>
-        <v>0.5</v>
-      </c>
-      <c r="C36" s="16" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="C36" s="15" t="n">
         <f aca="false">1-B36</f>
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="D36" s="10" t="n">
-        <f aca="false">SQRT( B36^2*B$4^2 + C36^2*C$4^2 + 2*B36*C36*B$6)</f>
-        <v>0.0400680945049446</v>
+        <f aca="false">SQRT( B36^2*B$4^2 + C36^2*C$4^2 + 2*B36*C36*B$7)</f>
+        <v>0.040626800790918</v>
       </c>
       <c r="E36" s="10" t="n">
         <f aca="false">B36*B$3 + C36*C$3</f>
-        <v>0.00717611536796452</v>
-      </c>
-      <c r="F36" s="18" t="n">
+        <v>0.00719523342621381</v>
+      </c>
+      <c r="F36" s="17" t="n">
         <f aca="false">E36/D36</f>
-        <v>0.179097994467367</v>
+        <v>0.177105587595819</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="1" t="n">
         <f aca="false">B36+0.02</f>
-        <v>0.52</v>
-      </c>
-      <c r="C37" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C37" s="15" t="n">
         <f aca="false">1-B37</f>
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="D37" s="10" t="n">
-        <f aca="false">SQRT( B37^2*B$4^2 + C37^2*C$4^2 + 2*B37*C37*B$6)</f>
-        <v>0.0395430478242518</v>
+        <f aca="false">SQRT( B37^2*B$4^2 + C37^2*C$4^2 + 2*B37*C37*B$7)</f>
+        <v>0.0400680945049446</v>
       </c>
       <c r="E37" s="10" t="n">
         <f aca="false">B37*B$3 + C37*C$3</f>
-        <v>0.00715699730971522</v>
-      </c>
-      <c r="F37" s="18" t="n">
+        <v>0.00717611536796452</v>
+      </c>
+      <c r="F37" s="17" t="n">
         <f aca="false">E37/D37</f>
-        <v>0.1809925563028</v>
+        <v>0.179097994467367</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="1" t="n">
         <f aca="false">B37+0.02</f>
-        <v>0.54</v>
-      </c>
-      <c r="C38" s="16" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="C38" s="15" t="n">
         <f aca="false">1-B38</f>
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="D38" s="10" t="n">
-        <f aca="false">SQRT( B38^2*B$4^2 + C38^2*C$4^2 + 2*B38*C38*B$6)</f>
-        <v>0.0390530183779258</v>
+        <f aca="false">SQRT( B38^2*B$4^2 + C38^2*C$4^2 + 2*B38*C38*B$7)</f>
+        <v>0.0395430478242518</v>
       </c>
       <c r="E38" s="10" t="n">
         <f aca="false">B38*B$3 + C38*C$3</f>
-        <v>0.00713787925146592</v>
-      </c>
-      <c r="F38" s="18" t="n">
+        <v>0.00715699730971522</v>
+      </c>
+      <c r="F38" s="17" t="n">
         <f aca="false">E38/D38</f>
-        <v>0.182774073501589</v>
+        <v>0.1809925563028</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="1" t="n">
         <f aca="false">B38+0.02</f>
-        <v>0.56</v>
-      </c>
-      <c r="C39" s="16" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="C39" s="15" t="n">
         <f aca="false">1-B39</f>
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="D39" s="10" t="n">
-        <f aca="false">SQRT( B39^2*B$4^2 + C39^2*C$4^2 + 2*B39*C39*B$6)</f>
-        <v>0.0385993398498447</v>
+        <f aca="false">SQRT( B39^2*B$4^2 + C39^2*C$4^2 + 2*B39*C39*B$7)</f>
+        <v>0.0390530183779258</v>
       </c>
       <c r="E39" s="10" t="n">
         <f aca="false">B39*B$3 + C39*C$3</f>
-        <v>0.00711876119321663</v>
-      </c>
-      <c r="F39" s="18" t="n">
+        <v>0.00713787925146592</v>
+      </c>
+      <c r="F39" s="17" t="n">
         <f aca="false">E39/D39</f>
-        <v>0.184427019242021</v>
+        <v>0.182774073501589</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="1" t="n">
         <f aca="false">B39+0.02</f>
-        <v>0.58</v>
-      </c>
-      <c r="C40" s="16" t="n">
+        <v>0.56</v>
+      </c>
+      <c r="C40" s="15" t="n">
         <f aca="false">1-B40</f>
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="D40" s="10" t="n">
-        <f aca="false">SQRT( B40^2*B$4^2 + C40^2*C$4^2 + 2*B40*C40*B$6)</f>
-        <v>0.0381833079824505</v>
+        <f aca="false">SQRT( B40^2*B$4^2 + C40^2*C$4^2 + 2*B40*C40*B$7)</f>
+        <v>0.0385993398498447</v>
       </c>
       <c r="E40" s="10" t="n">
         <f aca="false">B40*B$3 + C40*C$3</f>
-        <v>0.00709964313496733</v>
-      </c>
-      <c r="F40" s="18" t="n">
+        <v>0.00711876119321663</v>
+      </c>
+      <c r="F40" s="17" t="n">
         <f aca="false">E40/D40</f>
-        <v>0.185935779535665</v>
+        <v>0.184427019242021</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="1" t="n">
         <f aca="false">B40+0.02</f>
-        <v>0.6</v>
-      </c>
-      <c r="C41" s="16" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="C41" s="15" t="n">
         <f aca="false">1-B41</f>
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="D41" s="10" t="n">
-        <f aca="false">SQRT( B41^2*B$4^2 + C41^2*C$4^2 + 2*B41*C41*B$6)</f>
-        <v>0.0378061656260349</v>
+        <f aca="false">SQRT( B41^2*B$4^2 + C41^2*C$4^2 + 2*B41*C41*B$7)</f>
+        <v>0.0381833079824505</v>
       </c>
       <c r="E41" s="10" t="n">
         <f aca="false">B41*B$3 + C41*C$3</f>
-        <v>0.00708052507671803</v>
-      </c>
-      <c r="F41" s="18" t="n">
+        <v>0.00709964313496733</v>
+      </c>
+      <c r="F41" s="17" t="n">
         <f aca="false">E41/D41</f>
-        <v>0.18728492983806</v>
+        <v>0.185935779535665</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="1" t="n">
         <f aca="false">B41+0.02</f>
-        <v>0.62</v>
-      </c>
-      <c r="C42" s="16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C42" s="15" t="n">
         <f aca="false">1-B42</f>
-        <v>0.38</v>
+        <v>0.4</v>
       </c>
       <c r="D42" s="10" t="n">
-        <f aca="false">SQRT( B42^2*B$4^2 + C42^2*C$4^2 + 2*B42*C42*B$6)</f>
-        <v>0.0374690871175873</v>
+        <f aca="false">SQRT( B42^2*B$4^2 + C42^2*C$4^2 + 2*B42*C42*B$7)</f>
+        <v>0.0378061656260349</v>
       </c>
       <c r="E42" s="10" t="n">
         <f aca="false">B42*B$3 + C42*C$3</f>
-        <v>0.00706140701846874</v>
-      </c>
-      <c r="F42" s="18" t="n">
+        <v>0.00708052507671803</v>
+      </c>
+      <c r="F42" s="17" t="n">
         <f aca="false">E42/D42</f>
-        <v>0.188459542563935</v>
+        <v>0.18728492983806</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="1" t="n">
         <f aca="false">B42+0.02</f>
-        <v>0.64</v>
-      </c>
-      <c r="C43" s="16" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="C43" s="15" t="n">
         <f aca="false">1-B43</f>
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="D43" s="10" t="n">
-        <f aca="false">SQRT( B43^2*B$4^2 + C43^2*C$4^2 + 2*B43*C43*B$6)</f>
-        <v>0.0371731623450195</v>
+        <f aca="false">SQRT( B43^2*B$4^2 + C43^2*C$4^2 + 2*B43*C43*B$7)</f>
+        <v>0.0374690871175873</v>
       </c>
       <c r="E43" s="10" t="n">
         <f aca="false">B43*B$3 + C43*C$3</f>
-        <v>0.00704228896021944</v>
-      </c>
-      <c r="F43" s="18" t="n">
+        <v>0.00706140701846874</v>
+      </c>
+      <c r="F43" s="17" t="n">
         <f aca="false">E43/D43</f>
-        <v>0.189445517033419</v>
+        <v>0.188459542563935</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="1" t="n">
         <f aca="false">B43+0.02</f>
-        <v>0.66</v>
-      </c>
-      <c r="C44" s="16" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="C44" s="15" t="n">
         <f aca="false">1-B44</f>
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="D44" s="10" t="n">
-        <f aca="false">SQRT( B44^2*B$4^2 + C44^2*C$4^2 + 2*B44*C44*B$6)</f>
-        <v>0.0369193809164598</v>
+        <f aca="false">SQRT( B44^2*B$4^2 + C44^2*C$4^2 + 2*B44*C44*B$7)</f>
+        <v>0.0371731623450195</v>
       </c>
       <c r="E44" s="10" t="n">
         <f aca="false">B44*B$3 + C44*C$3</f>
-        <v>0.00702317090197014</v>
-      </c>
-      <c r="F44" s="18" t="n">
+        <v>0.00704228896021944</v>
+      </c>
+      <c r="F44" s="17" t="n">
         <f aca="false">E44/D44</f>
-        <v>0.190229920644173</v>
+        <v>0.189445517033419</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="1" t="n">
         <f aca="false">B44+0.02</f>
-        <v>0.68</v>
-      </c>
-      <c r="C45" s="16" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="C45" s="15" t="n">
         <f aca="false">1-B45</f>
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="D45" s="10" t="n">
-        <f aca="false">SQRT( B45^2*B$4^2 + C45^2*C$4^2 + 2*B45*C45*B$6)</f>
-        <v>0.0367086169039613</v>
+        <f aca="false">SQRT( B45^2*B$4^2 + C45^2*C$4^2 + 2*B45*C45*B$7)</f>
+        <v>0.0369193809164598</v>
       </c>
       <c r="E45" s="10" t="n">
         <f aca="false">B45*B$3 + C45*C$3</f>
-        <v>0.00700405284372084</v>
-      </c>
-      <c r="F45" s="18" t="n">
+        <v>0.00702317090197014</v>
+      </c>
+      <c r="F45" s="17" t="n">
         <f aca="false">E45/D45</f>
-        <v>0.190801327711288</v>
+        <v>0.190229920644173</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="1" t="n">
         <f aca="false">B45+0.02</f>
-        <v>0.7</v>
-      </c>
-      <c r="C46" s="16" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="C46" s="15" t="n">
         <f aca="false">1-B46</f>
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="D46" s="10" t="n">
-        <f aca="false">SQRT( B46^2*B$4^2 + C46^2*C$4^2 + 2*B46*C46*B$6)</f>
-        <v>0.0365416146601458</v>
+        <f aca="false">SQRT( B46^2*B$4^2 + C46^2*C$4^2 + 2*B46*C46*B$7)</f>
+        <v>0.0367086169039613</v>
       </c>
       <c r="E46" s="10" t="n">
         <f aca="false">B46*B$3 + C46*C$3</f>
+        <v>0.00700405284372084</v>
+      </c>
+      <c r="F46" s="17" t="n">
+        <f aca="false">E46/D46</f>
+        <v>0.190801327711288</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="1" t="n">
+        <f aca="false">B46+0.02</f>
+        <v>0.7</v>
+      </c>
+      <c r="C47" s="15" t="n">
+        <f aca="false">1-B47</f>
+        <v>0.3</v>
+      </c>
+      <c r="D47" s="10" t="n">
+        <f aca="false">SQRT( B47^2*B$4^2 + C47^2*C$4^2 + 2*B47*C47*B$7)</f>
+        <v>0.0365416146601458</v>
+      </c>
+      <c r="E47" s="10" t="n">
+        <f aca="false">B47*B$3 + C47*C$3</f>
         <v>0.00698493478547155</v>
       </c>
-      <c r="F46" s="18" t="n">
-        <f aca="false">E46/D46</f>
+      <c r="F47" s="17" t="n">
+        <f aca="false">E47/D47</f>
         <v>0.191150140748698</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="19" t="n">
-        <f aca="false">B46+0.02</f>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="18" t="n">
+        <f aca="false">B47+0.02</f>
         <v>0.72</v>
       </c>
-      <c r="C47" s="20" t="n">
-        <f aca="false">1-B47</f>
+      <c r="C48" s="19" t="n">
+        <f aca="false">1-B48</f>
         <v>0.28</v>
       </c>
-      <c r="D47" s="19" t="n">
-        <f aca="false">SQRT( B47^2*B$4^2 + C47^2*C$4^2 + 2*B47*C47*B$6)</f>
+      <c r="D48" s="18" t="n">
+        <f aca="false">SQRT( B48^2*B$4^2 + C48^2*C$4^2 + 2*B48*C48*B$7)</f>
         <v>0.0364189762096772</v>
       </c>
-      <c r="E47" s="19" t="n">
-        <f aca="false">B47*B$3 + C47*C$3</f>
+      <c r="E48" s="18" t="n">
+        <f aca="false">B48*B$3 + C48*C$3</f>
         <v>0.00696581672722225</v>
       </c>
-      <c r="F47" s="21" t="n">
-        <f aca="false">E47/D47</f>
+      <c r="F48" s="20" t="n">
+        <f aca="false">E48/D48</f>
         <v>0.191268878266032</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="1" t="n">
-        <f aca="false">B47+0.02</f>
-        <v>0.74</v>
-      </c>
-      <c r="C48" s="16" t="n">
-        <f aca="false">1-B48</f>
-        <v>0.26</v>
-      </c>
-      <c r="D48" s="10" t="n">
-        <f aca="false">SQRT( B48^2*B$4^2 + C48^2*C$4^2 + 2*B48*C48*B$6)</f>
-        <v>0.0363411506913738</v>
-      </c>
-      <c r="E48" s="10" t="n">
-        <f aca="false">B48*B$3 + C48*C$3</f>
-        <v>0.00694669866897295</v>
-      </c>
-      <c r="F48" s="18" t="n">
-        <f aca="false">E48/D48</f>
-        <v>0.1911524136362</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="1" t="n">
         <f aca="false">B48+0.02</f>
-        <v>0.76</v>
-      </c>
-      <c r="C49" s="16" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="C49" s="15" t="n">
         <f aca="false">1-B49</f>
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="D49" s="10" t="n">
-        <f aca="false">SQRT( B49^2*B$4^2 + C49^2*C$4^2 + 2*B49*C49*B$6)</f>
-        <v>0.0363084262700396</v>
+        <f aca="false">SQRT( B49^2*B$4^2 + C49^2*C$4^2 + 2*B49*C49*B$7)</f>
+        <v>0.0363411506913738</v>
       </c>
       <c r="E49" s="10" t="n">
         <f aca="false">B49*B$3 + C49*C$3</f>
-        <v>0.00692758061072366</v>
-      </c>
-      <c r="F49" s="18" t="n">
+        <v>0.00694669866897295</v>
+      </c>
+      <c r="F49" s="17" t="n">
         <f aca="false">E49/D49</f>
-        <v>0.190798151349238</v>
+        <v>0.1911524136362</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="1" t="n">
         <f aca="false">B49+0.02</f>
-        <v>0.78</v>
-      </c>
-      <c r="C50" s="16" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="C50" s="15" t="n">
         <f aca="false">1-B50</f>
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="D50" s="10" t="n">
-        <f aca="false">SQRT( B50^2*B$4^2 + C50^2*C$4^2 + 2*B50*C50*B$6)</f>
-        <v>0.0363209248514175</v>
+        <f aca="false">SQRT( B50^2*B$4^2 + C50^2*C$4^2 + 2*B50*C50*B$7)</f>
+        <v>0.0363084262700396</v>
       </c>
       <c r="E50" s="10" t="n">
         <f aca="false">B50*B$3 + C50*C$3</f>
-        <v>0.00690846255247436</v>
-      </c>
-      <c r="F50" s="18" t="n">
+        <v>0.00692758061072366</v>
+      </c>
+      <c r="F50" s="17" t="n">
         <f aca="false">E50/D50</f>
-        <v>0.190206129957749</v>
+        <v>0.190798151349238</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="1" t="n">
         <f aca="false">B50+0.02</f>
-        <v>0.8</v>
-      </c>
-      <c r="C51" s="16" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="C51" s="15" t="n">
         <f aca="false">1-B51</f>
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="D51" s="10" t="n">
-        <f aca="false">SQRT( B51^2*B$4^2 + C51^2*C$4^2 + 2*B51*C51*B$6)</f>
-        <v>0.0363785998237891</v>
+        <f aca="false">SQRT( B51^2*B$4^2 + C51^2*C$4^2 + 2*B51*C51*B$7)</f>
+        <v>0.0363209248514175</v>
       </c>
       <c r="E51" s="10" t="n">
         <f aca="false">B51*B$3 + C51*C$3</f>
-        <v>0.00688934449422506</v>
-      </c>
-      <c r="F51" s="18" t="n">
+        <v>0.00690846255247436</v>
+      </c>
+      <c r="F51" s="17" t="n">
         <f aca="false">E51/D51</f>
-        <v>0.189379045031851</v>
+        <v>0.190206129957749</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="1" t="n">
         <f aca="false">B51+0.02</f>
-        <v>0.82</v>
-      </c>
-      <c r="C52" s="16" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C52" s="15" t="n">
         <f aca="false">1-B52</f>
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="D52" s="10" t="n">
-        <f aca="false">SQRT( B52^2*B$4^2 + C52^2*C$4^2 + 2*B52*C52*B$6)</f>
-        <v>0.0364812369230831</v>
+        <f aca="false">SQRT( B52^2*B$4^2 + C52^2*C$4^2 + 2*B52*C52*B$7)</f>
+        <v>0.0363785998237891</v>
       </c>
       <c r="E52" s="10" t="n">
         <f aca="false">B52*B$3 + C52*C$3</f>
-        <v>0.00687022643597576</v>
-      </c>
-      <c r="F52" s="18" t="n">
+        <v>0.00688934449422506</v>
+      </c>
+      <c r="F52" s="17" t="n">
         <f aca="false">E52/D52</f>
-        <v>0.18832219012916</v>
+        <v>0.189379045031851</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="1" t="n">
         <f aca="false">B52+0.02</f>
-        <v>0.84</v>
-      </c>
-      <c r="C53" s="16" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="C53" s="15" t="n">
         <f aca="false">1-B53</f>
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="D53" s="10" t="n">
-        <f aca="false">SQRT( B53^2*B$4^2 + C53^2*C$4^2 + 2*B53*C53*B$6)</f>
-        <v>0.036628458184293</v>
+        <f aca="false">SQRT( B53^2*B$4^2 + C53^2*C$4^2 + 2*B53*C53*B$7)</f>
+        <v>0.0364812369230831</v>
       </c>
       <c r="E53" s="10" t="n">
         <f aca="false">B53*B$3 + C53*C$3</f>
-        <v>0.00685110837772647</v>
-      </c>
-      <c r="F53" s="18" t="n">
+        <v>0.00687022643597576</v>
+      </c>
+      <c r="F53" s="17" t="n">
         <f aca="false">E53/D53</f>
-        <v>0.187043318701969</v>
+        <v>0.18832219012916</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="1" t="n">
         <f aca="false">B53+0.02</f>
-        <v>0.86</v>
-      </c>
-      <c r="C54" s="16" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="C54" s="15" t="n">
         <f aca="false">1-B54</f>
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="D54" s="10" t="n">
-        <f aca="false">SQRT( B54^2*B$4^2 + C54^2*C$4^2 + 2*B54*C54*B$6)</f>
-        <v>0.0368197288107958</v>
+        <f aca="false">SQRT( B54^2*B$4^2 + C54^2*C$4^2 + 2*B54*C54*B$7)</f>
+        <v>0.036628458184293</v>
       </c>
       <c r="E54" s="10" t="n">
         <f aca="false">B54*B$3 + C54*C$3</f>
-        <v>0.00683199031947717</v>
-      </c>
-      <c r="F54" s="18" t="n">
+        <v>0.00685110837772647</v>
+      </c>
+      <c r="F54" s="17" t="n">
         <f aca="false">E54/D54</f>
-        <v>0.185552434527274</v>
+        <v>0.187043318701969</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="1" t="n">
         <f aca="false">B54+0.02</f>
-        <v>0.88</v>
-      </c>
-      <c r="C55" s="16" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="C55" s="15" t="n">
         <f aca="false">1-B55</f>
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="D55" s="10" t="n">
-        <f aca="false">SQRT( B55^2*B$4^2 + C55^2*C$4^2 + 2*B55*C55*B$6)</f>
-        <v>0.0370543666747151</v>
+        <f aca="false">SQRT( B55^2*B$4^2 + C55^2*C$4^2 + 2*B55*C55*B$7)</f>
+        <v>0.0368197288107958</v>
       </c>
       <c r="E55" s="10" t="n">
         <f aca="false">B55*B$3 + C55*C$3</f>
-        <v>0.00681287226122787</v>
-      </c>
-      <c r="F55" s="18" t="n">
+        <v>0.00683199031947717</v>
+      </c>
+      <c r="F55" s="17" t="n">
         <f aca="false">E55/D55</f>
-        <v>0.183861522206957</v>
+        <v>0.185552434527274</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="1" t="n">
         <f aca="false">B55+0.02</f>
-        <v>0.900000000000001</v>
-      </c>
-      <c r="C56" s="16" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="C56" s="15" t="n">
         <f aca="false">1-B56</f>
-        <v>0.0999999999999995</v>
+        <v>0.12</v>
       </c>
       <c r="D56" s="10" t="n">
-        <f aca="false">SQRT( B56^2*B$4^2 + C56^2*C$4^2 + 2*B56*C56*B$6)</f>
-        <v>0.0373315540642175</v>
+        <f aca="false">SQRT( B56^2*B$4^2 + C56^2*C$4^2 + 2*B56*C56*B$7)</f>
+        <v>0.0370543666747151</v>
       </c>
       <c r="E56" s="10" t="n">
         <f aca="false">B56*B$3 + C56*C$3</f>
-        <v>0.00679375420297858</v>
-      </c>
-      <c r="F56" s="18" t="n">
+        <v>0.00681287226122787</v>
+      </c>
+      <c r="F56" s="17" t="n">
         <f aca="false">E56/D56</f>
-        <v>0.181984232193817</v>
+        <v>0.183861522206957</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="1" t="n">
         <f aca="false">B56+0.02</f>
-        <v>0.920000000000001</v>
-      </c>
-      <c r="C57" s="16" t="n">
+        <v>0.900000000000001</v>
+      </c>
+      <c r="C57" s="15" t="n">
         <f aca="false">1-B57</f>
-        <v>0.0799999999999995</v>
+        <v>0.0999999999999995</v>
       </c>
       <c r="D57" s="10" t="n">
-        <f aca="false">SQRT( B57^2*B$4^2 + C57^2*C$4^2 + 2*B57*C57*B$6)</f>
-        <v>0.037650351223549</v>
+        <f aca="false">SQRT( B57^2*B$4^2 + C57^2*C$4^2 + 2*B57*C57*B$7)</f>
+        <v>0.0373315540642175</v>
       </c>
       <c r="E57" s="10" t="n">
         <f aca="false">B57*B$3 + C57*C$3</f>
-        <v>0.00677463614472928</v>
-      </c>
-      <c r="F57" s="18" t="n">
+        <v>0.00679375420297858</v>
+      </c>
+      <c r="F57" s="17" t="n">
         <f aca="false">E57/D57</f>
-        <v>0.179935536444398</v>
+        <v>0.181984232193817</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="1" t="n">
         <f aca="false">B57+0.02</f>
-        <v>0.940000000000001</v>
-      </c>
-      <c r="C58" s="16" t="n">
+        <v>0.920000000000001</v>
+      </c>
+      <c r="C58" s="15" t="n">
         <f aca="false">1-B58</f>
-        <v>0.0599999999999995</v>
+        <v>0.0799999999999995</v>
       </c>
       <c r="D58" s="10" t="n">
-        <f aca="false">SQRT( B58^2*B$4^2 + C58^2*C$4^2 + 2*B58*C58*B$6)</f>
-        <v>0.038009711191816</v>
+        <f aca="false">SQRT( B58^2*B$4^2 + C58^2*C$4^2 + 2*B58*C58*B$7)</f>
+        <v>0.037650351223549</v>
       </c>
       <c r="E58" s="10" t="n">
         <f aca="false">B58*B$3 + C58*C$3</f>
-        <v>0.00675551808647998</v>
-      </c>
-      <c r="F58" s="18" t="n">
+        <v>0.00677463614472928</v>
+      </c>
+      <c r="F58" s="17" t="n">
         <f aca="false">E58/D58</f>
-        <v>0.177731371132715</v>
+        <v>0.179935536444398</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="1" t="n">
         <f aca="false">B58+0.02</f>
-        <v>0.960000000000001</v>
-      </c>
-      <c r="C59" s="16" t="n">
+        <v>0.940000000000001</v>
+      </c>
+      <c r="C59" s="15" t="n">
         <f aca="false">1-B59</f>
-        <v>0.0399999999999995</v>
+        <v>0.0599999999999995</v>
       </c>
       <c r="D59" s="10" t="n">
-        <f aca="false">SQRT( B59^2*B$4^2 + C59^2*C$4^2 + 2*B59*C59*B$6)</f>
-        <v>0.03840849543702</v>
+        <f aca="false">SQRT( B59^2*B$4^2 + C59^2*C$4^2 + 2*B59*C59*B$7)</f>
+        <v>0.038009711191816</v>
       </c>
       <c r="E59" s="10" t="n">
         <f aca="false">B59*B$3 + C59*C$3</f>
-        <v>0.00673640002823068</v>
-      </c>
-      <c r="F59" s="18" t="n">
+        <v>0.00675551808647998</v>
+      </c>
+      <c r="F59" s="17" t="n">
         <f aca="false">E59/D59</f>
-        <v>0.175388281982475</v>
+        <v>0.177731371132715</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="1" t="n">
         <f aca="false">B59+0.02</f>
-        <v>0.980000000000001</v>
-      </c>
-      <c r="C60" s="16" t="n">
+        <v>0.960000000000001</v>
+      </c>
+      <c r="C60" s="15" t="n">
         <f aca="false">1-B60</f>
-        <v>0.0199999999999995</v>
+        <v>0.0399999999999995</v>
       </c>
       <c r="D60" s="10" t="n">
-        <f aca="false">SQRT( B60^2*B$4^2 + C60^2*C$4^2 + 2*B60*C60*B$6)</f>
-        <v>0.0388454898000728</v>
+        <f aca="false">SQRT( B60^2*B$4^2 + C60^2*C$4^2 + 2*B60*C60*B$7)</f>
+        <v>0.03840849543702</v>
       </c>
       <c r="E60" s="10" t="n">
         <f aca="false">B60*B$3 + C60*C$3</f>
-        <v>0.00671728196998139</v>
-      </c>
-      <c r="F60" s="18" t="n">
+        <v>0.00673640002823068</v>
+      </c>
+      <c r="F60" s="17" t="n">
         <f aca="false">E60/D60</f>
-        <v>0.172923085911734</v>
+        <v>0.175388281982475</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="1" t="n">
         <f aca="false">B60+0.02</f>
-        <v>1</v>
-      </c>
-      <c r="C61" s="16" t="n">
+        <v>0.980000000000001</v>
+      </c>
+      <c r="C61" s="15" t="n">
         <f aca="false">1-B61</f>
-        <v>0</v>
+        <v>0.0199999999999995</v>
       </c>
       <c r="D61" s="10" t="n">
-        <f aca="false">SQRT( B61^2*B$4^2 + C61^2*C$4^2 + 2*B61*C61*B$6)</f>
-        <v>0.039319420304745</v>
+        <f aca="false">SQRT( B61^2*B$4^2 + C61^2*C$4^2 + 2*B61*C61*B$7)</f>
+        <v>0.0388454898000728</v>
       </c>
       <c r="E61" s="10" t="n">
         <f aca="false">B61*B$3 + C61*C$3</f>
-        <v>0.00669816391173209</v>
-      </c>
-      <c r="F61" s="18" t="n">
+        <v>0.00671728196998139</v>
+      </c>
+      <c r="F61" s="17" t="n">
         <f aca="false">E61/D61</f>
-        <v>0.170352560129778</v>
+        <v>0.172923085911734</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="1" t="n">
         <f aca="false">B61+0.02</f>
-        <v>1.02</v>
-      </c>
-      <c r="C62" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="15" t="n">
         <f aca="false">1-B62</f>
-        <v>-0.0200000000000005</v>
+        <v>0</v>
       </c>
       <c r="D62" s="10" t="n">
-        <f aca="false">SQRT( B62^2*B$4^2 + C62^2*C$4^2 + 2*B62*C62*B$6)</f>
-        <v>0.039828968447808</v>
+        <f aca="false">SQRT( B62^2*B$4^2 + C62^2*C$4^2 + 2*B62*C62*B$7)</f>
+        <v>0.039319420304745</v>
       </c>
       <c r="E62" s="10" t="n">
         <f aca="false">B62*B$3 + C62*C$3</f>
+        <v>0.00669816391173209</v>
+      </c>
+      <c r="F62" s="17" t="n">
+        <f aca="false">E62/D62</f>
+        <v>0.170352560129778</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="1" t="n">
+        <f aca="false">B62+0.02</f>
+        <v>1.02</v>
+      </c>
+      <c r="C63" s="15" t="n">
+        <f aca="false">1-B63</f>
+        <v>-0.0200000000000005</v>
+      </c>
+      <c r="D63" s="10" t="n">
+        <f aca="false">SQRT( B63^2*B$4^2 + C63^2*C$4^2 + 2*B63*C63*B$7)</f>
+        <v>0.039828968447808</v>
+      </c>
+      <c r="E63" s="10" t="n">
+        <f aca="false">B63*B$3 + C63*C$3</f>
         <v>0.00667904585348279</v>
       </c>
-      <c r="F62" s="18" t="n">
-        <f aca="false">E62/D62</f>
+      <c r="F63" s="17" t="n">
+        <f aca="false">E63/D63</f>
         <v>0.167693166902754</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="14" t="s">
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E68" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F68" s="16" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C67" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D67" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="E67" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="F67" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="G67" s="22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B68" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C68" s="10" t="n">
-        <f aca="false">1-B68</f>
-        <v>1</v>
-      </c>
-      <c r="D68" s="10" t="n">
-        <f aca="false">B68*D$47</f>
-        <v>0</v>
-      </c>
-      <c r="E68" s="10" t="n">
-        <f aca="false">B68*E$47</f>
-        <v>0</v>
-      </c>
-      <c r="F68" s="18" t="e">
-        <f aca="false">E68/D68</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G68" s="22" t="n">
-        <f aca="false">E68-0.5*8*D68^2</f>
-        <v>0</v>
+      <c r="G68" s="21" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="10" t="n">
-        <f aca="false">B68+0.02</f>
-        <v>0.02</v>
+      <c r="B69" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="C69" s="10" t="n">
         <f aca="false">1-B69</f>
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="D69" s="10" t="n">
-        <f aca="false">B69*D$47</f>
-        <v>0.000728379524193544</v>
+        <f aca="false">B69*D$48</f>
+        <v>0</v>
       </c>
       <c r="E69" s="10" t="n">
-        <f aca="false">B69*E$47</f>
-        <v>0.000139316334544445</v>
-      </c>
-      <c r="F69" s="18" t="n">
+        <f aca="false">B69*E$48</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="17" t="e">
         <f aca="false">E69/D69</f>
-        <v>0.191268878266032</v>
-      </c>
-      <c r="G69" s="22" t="n">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G69" s="21" t="n">
         <f aca="false">E69-0.5*8*D69^2</f>
-        <v>0.000137194187619387</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="10" t="n">
         <f aca="false">B69+0.02</f>
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="C70" s="10" t="n">
         <f aca="false">1-B70</f>
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="D70" s="10" t="n">
-        <f aca="false">B70*D$47</f>
-        <v>0.00145675904838709</v>
+        <f aca="false">B70*D$48</f>
+        <v>0.000728379524193544</v>
       </c>
       <c r="E70" s="10" t="n">
-        <f aca="false">B70*E$47</f>
-        <v>0.00027863266908889</v>
-      </c>
-      <c r="F70" s="18" t="n">
+        <f aca="false">B70*E$48</f>
+        <v>0.000139316334544445</v>
+      </c>
+      <c r="F70" s="17" t="n">
         <f aca="false">E70/D70</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G70" s="22" t="n">
+      <c r="G70" s="21" t="n">
         <f aca="false">E70-0.5*8*D70^2</f>
-        <v>0.000270144081388659</v>
+        <v>0.000137194187619387</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="10" t="n">
         <f aca="false">B70+0.02</f>
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="C71" s="10" t="n">
         <f aca="false">1-B71</f>
-        <v>0.94</v>
+        <v>0.96</v>
       </c>
       <c r="D71" s="10" t="n">
-        <f aca="false">B71*D$47</f>
-        <v>0.00218513857258063</v>
+        <f aca="false">B71*D$48</f>
+        <v>0.00145675904838709</v>
       </c>
       <c r="E71" s="10" t="n">
-        <f aca="false">B71*E$47</f>
-        <v>0.000417949003633335</v>
-      </c>
-      <c r="F71" s="18" t="n">
+        <f aca="false">B71*E$48</f>
+        <v>0.00027863266908889</v>
+      </c>
+      <c r="F71" s="17" t="n">
         <f aca="false">E71/D71</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G71" s="22" t="n">
+      <c r="G71" s="21" t="n">
         <f aca="false">E71-0.5*8*D71^2</f>
-        <v>0.000398849681307816</v>
+        <v>0.000270144081388659</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="10" t="n">
         <f aca="false">B71+0.02</f>
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="C72" s="10" t="n">
         <f aca="false">1-B72</f>
-        <v>0.92</v>
+        <v>0.94</v>
       </c>
       <c r="D72" s="10" t="n">
-        <f aca="false">B72*D$47</f>
-        <v>0.00291351809677418</v>
+        <f aca="false">B72*D$48</f>
+        <v>0.00218513857258063</v>
       </c>
       <c r="E72" s="10" t="n">
-        <f aca="false">B72*E$47</f>
-        <v>0.00055726533817778</v>
-      </c>
-      <c r="F72" s="18" t="n">
+        <f aca="false">B72*E$48</f>
+        <v>0.000417949003633335</v>
+      </c>
+      <c r="F72" s="17" t="n">
         <f aca="false">E72/D72</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G72" s="22" t="n">
+      <c r="G72" s="21" t="n">
         <f aca="false">E72-0.5*8*D72^2</f>
-        <v>0.000523310987376858</v>
+        <v>0.000398849681307816</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="10" t="n">
         <f aca="false">B72+0.02</f>
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="C73" s="10" t="n">
         <f aca="false">1-B73</f>
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="D73" s="10" t="n">
-        <f aca="false">B73*D$47</f>
-        <v>0.00364189762096772</v>
+        <f aca="false">B73*D$48</f>
+        <v>0.00291351809677418</v>
       </c>
       <c r="E73" s="10" t="n">
-        <f aca="false">B73*E$47</f>
-        <v>0.000696581672722225</v>
-      </c>
-      <c r="F73" s="18" t="n">
+        <f aca="false">B73*E$48</f>
+        <v>0.00055726533817778</v>
+      </c>
+      <c r="F73" s="17" t="n">
         <f aca="false">E73/D73</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G73" s="22" t="n">
+      <c r="G73" s="21" t="n">
         <f aca="false">E73-0.5*8*D73^2</f>
-        <v>0.000643527999595784</v>
+        <v>0.000523310987376858</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="10" t="n">
         <f aca="false">B73+0.02</f>
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="C74" s="10" t="n">
         <f aca="false">1-B74</f>
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="D74" s="10" t="n">
-        <f aca="false">B74*D$47</f>
-        <v>0.00437027714516127</v>
+        <f aca="false">B74*D$48</f>
+        <v>0.00364189762096772</v>
       </c>
       <c r="E74" s="10" t="n">
-        <f aca="false">B74*E$47</f>
-        <v>0.00083589800726667</v>
-      </c>
-      <c r="F74" s="18" t="n">
+        <f aca="false">B74*E$48</f>
+        <v>0.000696581672722225</v>
+      </c>
+      <c r="F74" s="17" t="n">
         <f aca="false">E74/D74</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G74" s="22" t="n">
+      <c r="G74" s="21" t="n">
         <f aca="false">E74-0.5*8*D74^2</f>
-        <v>0.000759500717964594</v>
+        <v>0.000643527999595784</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="10" t="n">
         <f aca="false">B74+0.02</f>
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="C75" s="10" t="n">
         <f aca="false">1-B75</f>
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="D75" s="10" t="n">
-        <f aca="false">B75*D$47</f>
-        <v>0.00509865666935481</v>
+        <f aca="false">B75*D$48</f>
+        <v>0.00437027714516127</v>
       </c>
       <c r="E75" s="10" t="n">
-        <f aca="false">B75*E$47</f>
-        <v>0.000975214341811115</v>
-      </c>
-      <c r="F75" s="18" t="n">
+        <f aca="false">B75*E$48</f>
+        <v>0.00083589800726667</v>
+      </c>
+      <c r="F75" s="17" t="n">
         <f aca="false">E75/D75</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G75" s="22" t="n">
+      <c r="G75" s="21" t="n">
         <f aca="false">E75-0.5*8*D75^2</f>
-        <v>0.00087122914248329</v>
+        <v>0.000759500717964594</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="10" t="n">
         <f aca="false">B75+0.02</f>
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="C76" s="10" t="n">
         <f aca="false">1-B76</f>
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="D76" s="10" t="n">
-        <f aca="false">B76*D$47</f>
-        <v>0.00582703619354835</v>
+        <f aca="false">B76*D$48</f>
+        <v>0.00509865666935481</v>
       </c>
       <c r="E76" s="10" t="n">
-        <f aca="false">B76*E$47</f>
-        <v>0.00111453067635556</v>
-      </c>
-      <c r="F76" s="18" t="n">
+        <f aca="false">B76*E$48</f>
+        <v>0.000975214341811115</v>
+      </c>
+      <c r="F76" s="17" t="n">
         <f aca="false">E76/D76</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G76" s="22" t="n">
+      <c r="G76" s="21" t="n">
         <f aca="false">E76-0.5*8*D76^2</f>
-        <v>0.00097871327315187</v>
+        <v>0.00087122914248329</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="10" t="n">
         <f aca="false">B76+0.02</f>
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="C77" s="10" t="n">
         <f aca="false">1-B77</f>
-        <v>0.82</v>
+        <v>0.84</v>
       </c>
       <c r="D77" s="10" t="n">
-        <f aca="false">B77*D$47</f>
-        <v>0.0065554157177419</v>
+        <f aca="false">B77*D$48</f>
+        <v>0.00582703619354835</v>
       </c>
       <c r="E77" s="10" t="n">
-        <f aca="false">B77*E$47</f>
-        <v>0.0012538470109</v>
-      </c>
-      <c r="F77" s="18" t="n">
+        <f aca="false">B77*E$48</f>
+        <v>0.00111453067635556</v>
+      </c>
+      <c r="F77" s="17" t="n">
         <f aca="false">E77/D77</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G77" s="22" t="n">
+      <c r="G77" s="21" t="n">
         <f aca="false">E77-0.5*8*D77^2</f>
-        <v>0.00108195310997033</v>
+        <v>0.00097871327315187</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="10" t="n">
         <f aca="false">B77+0.02</f>
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="C78" s="10" t="n">
         <f aca="false">1-B78</f>
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="D78" s="10" t="n">
-        <f aca="false">B78*D$47</f>
-        <v>0.00728379524193544</v>
+        <f aca="false">B78*D$48</f>
+        <v>0.0065554157177419</v>
       </c>
       <c r="E78" s="10" t="n">
-        <f aca="false">B78*E$47</f>
-        <v>0.00139316334544445</v>
-      </c>
-      <c r="F78" s="18" t="n">
+        <f aca="false">B78*E$48</f>
+        <v>0.0012538470109</v>
+      </c>
+      <c r="F78" s="17" t="n">
         <f aca="false">E78/D78</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G78" s="22" t="n">
+      <c r="G78" s="21" t="n">
         <f aca="false">E78-0.5*8*D78^2</f>
-        <v>0.00118094865293868</v>
+        <v>0.00108195310997033</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="10" t="n">
         <f aca="false">B78+0.02</f>
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="C79" s="10" t="n">
         <f aca="false">1-B79</f>
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="D79" s="10" t="n">
-        <f aca="false">B79*D$47</f>
-        <v>0.00801217476612899</v>
+        <f aca="false">B79*D$48</f>
+        <v>0.00728379524193544</v>
       </c>
       <c r="E79" s="10" t="n">
-        <f aca="false">B79*E$47</f>
-        <v>0.00153247967998889</v>
-      </c>
-      <c r="F79" s="18" t="n">
+        <f aca="false">B79*E$48</f>
+        <v>0.00139316334544445</v>
+      </c>
+      <c r="F79" s="17" t="n">
         <f aca="false">E79/D79</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G79" s="22" t="n">
+      <c r="G79" s="21" t="n">
         <f aca="false">E79-0.5*8*D79^2</f>
-        <v>0.00127569990205692</v>
+        <v>0.00118094865293868</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="10" t="n">
         <f aca="false">B79+0.02</f>
-        <v>0.24</v>
+        <v>0.22</v>
       </c>
       <c r="C80" s="10" t="n">
         <f aca="false">1-B80</f>
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="D80" s="10" t="n">
-        <f aca="false">B80*D$47</f>
-        <v>0.00874055429032253</v>
+        <f aca="false">B80*D$48</f>
+        <v>0.00801217476612899</v>
       </c>
       <c r="E80" s="10" t="n">
-        <f aca="false">B80*E$47</f>
-        <v>0.00167179601453334</v>
-      </c>
-      <c r="F80" s="18" t="n">
+        <f aca="false">B80*E$48</f>
+        <v>0.00153247967998889</v>
+      </c>
+      <c r="F80" s="17" t="n">
         <f aca="false">E80/D80</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G80" s="22" t="n">
+      <c r="G80" s="21" t="n">
         <f aca="false">E80-0.5*8*D80^2</f>
-        <v>0.00136620685732504</v>
+        <v>0.00127569990205692</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="10" t="n">
         <f aca="false">B80+0.02</f>
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="C81" s="10" t="n">
         <f aca="false">1-B81</f>
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="D81" s="10" t="n">
-        <f aca="false">B81*D$47</f>
-        <v>0.00946893381451607</v>
+        <f aca="false">B81*D$48</f>
+        <v>0.00874055429032253</v>
       </c>
       <c r="E81" s="10" t="n">
-        <f aca="false">B81*E$47</f>
-        <v>0.00181111234907778</v>
-      </c>
-      <c r="F81" s="18" t="n">
+        <f aca="false">B81*E$48</f>
+        <v>0.00167179601453334</v>
+      </c>
+      <c r="F81" s="17" t="n">
         <f aca="false">E81/D81</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G81" s="22" t="n">
+      <c r="G81" s="21" t="n">
         <f aca="false">E81-0.5*8*D81^2</f>
-        <v>0.00145246951874304</v>
+        <v>0.00136620685732504</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="10" t="n">
         <f aca="false">B81+0.02</f>
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
       <c r="C82" s="10" t="n">
         <f aca="false">1-B82</f>
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="D82" s="10" t="n">
-        <f aca="false">B82*D$47</f>
-        <v>0.0101973133387096</v>
+        <f aca="false">B82*D$48</f>
+        <v>0.00946893381451607</v>
       </c>
       <c r="E82" s="10" t="n">
-        <f aca="false">B82*E$47</f>
-        <v>0.00195042868362223</v>
-      </c>
-      <c r="F82" s="18" t="n">
+        <f aca="false">B82*E$48</f>
+        <v>0.00181111234907778</v>
+      </c>
+      <c r="F82" s="17" t="n">
         <f aca="false">E82/D82</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G82" s="22" t="n">
+      <c r="G82" s="21" t="n">
         <f aca="false">E82-0.5*8*D82^2</f>
-        <v>0.00153448788631093</v>
+        <v>0.00145246951874304</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="10" t="n">
         <f aca="false">B82+0.02</f>
-        <v>0.3</v>
+        <v>0.28</v>
       </c>
       <c r="C83" s="10" t="n">
         <f aca="false">1-B83</f>
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="D83" s="10" t="n">
-        <f aca="false">B83*D$47</f>
-        <v>0.0109256928629032</v>
+        <f aca="false">B83*D$48</f>
+        <v>0.0101973133387096</v>
       </c>
       <c r="E83" s="10" t="n">
-        <f aca="false">B83*E$47</f>
-        <v>0.00208974501816668</v>
-      </c>
-      <c r="F83" s="18" t="n">
+        <f aca="false">B83*E$48</f>
+        <v>0.00195042868362223</v>
+      </c>
+      <c r="F83" s="17" t="n">
         <f aca="false">E83/D83</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G83" s="22" t="n">
+      <c r="G83" s="21" t="n">
         <f aca="false">E83-0.5*8*D83^2</f>
-        <v>0.0016122619600287</v>
+        <v>0.00153448788631093</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="10" t="n">
         <f aca="false">B83+0.02</f>
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="C84" s="10" t="n">
         <f aca="false">1-B84</f>
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
       <c r="D84" s="10" t="n">
-        <f aca="false">B84*D$47</f>
-        <v>0.0116540723870967</v>
+        <f aca="false">B84*D$48</f>
+        <v>0.0109256928629032</v>
       </c>
       <c r="E84" s="10" t="n">
-        <f aca="false">B84*E$47</f>
-        <v>0.00222906135271112</v>
-      </c>
-      <c r="F84" s="18" t="n">
+        <f aca="false">B84*E$48</f>
+        <v>0.00208974501816668</v>
+      </c>
+      <c r="F84" s="17" t="n">
         <f aca="false">E84/D84</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G84" s="22" t="n">
+      <c r="G84" s="21" t="n">
         <f aca="false">E84-0.5*8*D84^2</f>
-        <v>0.00168579173989636</v>
+        <v>0.0016122619600287</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="10" t="n">
         <f aca="false">B84+0.02</f>
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="C85" s="10" t="n">
         <f aca="false">1-B85</f>
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="D85" s="10" t="n">
-        <f aca="false">B85*D$47</f>
-        <v>0.0123824519112903</v>
+        <f aca="false">B85*D$48</f>
+        <v>0.0116540723870967</v>
       </c>
       <c r="E85" s="10" t="n">
-        <f aca="false">B85*E$47</f>
-        <v>0.00236837768725557</v>
-      </c>
-      <c r="F85" s="18" t="n">
+        <f aca="false">B85*E$48</f>
+        <v>0.00222906135271112</v>
+      </c>
+      <c r="F85" s="17" t="n">
         <f aca="false">E85/D85</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G85" s="22" t="n">
+      <c r="G85" s="21" t="n">
         <f aca="false">E85-0.5*8*D85^2</f>
-        <v>0.0017550772259139</v>
+        <v>0.00168579173989636</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="10" t="n">
         <f aca="false">B85+0.02</f>
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="C86" s="10" t="n">
         <f aca="false">1-B86</f>
-        <v>0.64</v>
+        <v>0.66</v>
       </c>
       <c r="D86" s="10" t="n">
-        <f aca="false">B86*D$47</f>
-        <v>0.0131108314354838</v>
+        <f aca="false">B86*D$48</f>
+        <v>0.0123824519112903</v>
       </c>
       <c r="E86" s="10" t="n">
-        <f aca="false">B86*E$47</f>
-        <v>0.00250769402180001</v>
-      </c>
-      <c r="F86" s="18" t="n">
+        <f aca="false">B86*E$48</f>
+        <v>0.00236837768725557</v>
+      </c>
+      <c r="F86" s="17" t="n">
         <f aca="false">E86/D86</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G86" s="22" t="n">
+      <c r="G86" s="21" t="n">
         <f aca="false">E86-0.5*8*D86^2</f>
-        <v>0.00182011841808133</v>
+        <v>0.0017550772259139</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="10" t="n">
         <f aca="false">B86+0.02</f>
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="C87" s="10" t="n">
         <f aca="false">1-B87</f>
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
       <c r="D87" s="10" t="n">
-        <f aca="false">B87*D$47</f>
-        <v>0.0138392109596773</v>
+        <f aca="false">B87*D$48</f>
+        <v>0.0131108314354838</v>
       </c>
       <c r="E87" s="10" t="n">
-        <f aca="false">B87*E$47</f>
-        <v>0.00264701035634446</v>
-      </c>
-      <c r="F87" s="18" t="n">
+        <f aca="false">B87*E$48</f>
+        <v>0.00250769402180001</v>
+      </c>
+      <c r="F87" s="17" t="n">
         <f aca="false">E87/D87</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G87" s="22" t="n">
+      <c r="G87" s="21" t="n">
         <f aca="false">E87-0.5*8*D87^2</f>
-        <v>0.00188091531639864</v>
+        <v>0.00182011841808133</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="10" t="n">
         <f aca="false">B87+0.02</f>
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="C88" s="10" t="n">
         <f aca="false">1-B88</f>
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="D88" s="10" t="n">
-        <f aca="false">B88*D$47</f>
-        <v>0.0145675904838709</v>
+        <f aca="false">B88*D$48</f>
+        <v>0.0138392109596773</v>
       </c>
       <c r="E88" s="10" t="n">
-        <f aca="false">B88*E$47</f>
-        <v>0.0027863266908889</v>
-      </c>
-      <c r="F88" s="18" t="n">
+        <f aca="false">B88*E$48</f>
+        <v>0.00264701035634446</v>
+      </c>
+      <c r="F88" s="17" t="n">
         <f aca="false">E88/D88</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G88" s="22" t="n">
+      <c r="G88" s="21" t="n">
         <f aca="false">E88-0.5*8*D88^2</f>
-        <v>0.00193746792086584</v>
+        <v>0.00188091531639864</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="10" t="n">
         <f aca="false">B88+0.02</f>
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="C89" s="10" t="n">
         <f aca="false">1-B89</f>
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="D89" s="10" t="n">
-        <f aca="false">B89*D$47</f>
-        <v>0.0152959700080644</v>
+        <f aca="false">B89*D$48</f>
+        <v>0.0145675904838709</v>
       </c>
       <c r="E89" s="10" t="n">
-        <f aca="false">B89*E$47</f>
-        <v>0.00292564302543335</v>
-      </c>
-      <c r="F89" s="18" t="n">
+        <f aca="false">B89*E$48</f>
+        <v>0.0027863266908889</v>
+      </c>
+      <c r="F89" s="17" t="n">
         <f aca="false">E89/D89</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G89" s="22" t="n">
+      <c r="G89" s="21" t="n">
         <f aca="false">E89-0.5*8*D89^2</f>
-        <v>0.00198977623148292</v>
+        <v>0.00193746792086584</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="10" t="n">
         <f aca="false">B89+0.02</f>
-        <v>0.44</v>
+        <v>0.42</v>
       </c>
       <c r="C90" s="10" t="n">
         <f aca="false">1-B90</f>
-        <v>0.56</v>
+        <v>0.58</v>
       </c>
       <c r="D90" s="10" t="n">
-        <f aca="false">B90*D$47</f>
-        <v>0.016024349532258</v>
+        <f aca="false">B90*D$48</f>
+        <v>0.0152959700080644</v>
       </c>
       <c r="E90" s="10" t="n">
-        <f aca="false">B90*E$47</f>
-        <v>0.00306495935997779</v>
-      </c>
-      <c r="F90" s="18" t="n">
+        <f aca="false">B90*E$48</f>
+        <v>0.00292564302543335</v>
+      </c>
+      <c r="F90" s="17" t="n">
         <f aca="false">E90/D90</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G90" s="22" t="n">
+      <c r="G90" s="21" t="n">
         <f aca="false">E90-0.5*8*D90^2</f>
-        <v>0.00203784024824988</v>
+        <v>0.00198977623148292</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="10" t="n">
         <f aca="false">B90+0.02</f>
-        <v>0.46</v>
+        <v>0.44</v>
       </c>
       <c r="C91" s="10" t="n">
         <f aca="false">1-B91</f>
-        <v>0.54</v>
+        <v>0.56</v>
       </c>
       <c r="D91" s="10" t="n">
-        <f aca="false">B91*D$47</f>
-        <v>0.0167527290564515</v>
+        <f aca="false">B91*D$48</f>
+        <v>0.016024349532258</v>
       </c>
       <c r="E91" s="10" t="n">
-        <f aca="false">B91*E$47</f>
-        <v>0.00320427569452224</v>
-      </c>
-      <c r="F91" s="18" t="n">
+        <f aca="false">B91*E$48</f>
+        <v>0.00306495935997779</v>
+      </c>
+      <c r="F91" s="17" t="n">
         <f aca="false">E91/D91</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G91" s="22" t="n">
+      <c r="G91" s="21" t="n">
         <f aca="false">E91-0.5*8*D91^2</f>
-        <v>0.00208165997116674</v>
+        <v>0.00203784024824988</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="10" t="n">
         <f aca="false">B91+0.02</f>
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="C92" s="10" t="n">
         <f aca="false">1-B92</f>
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="D92" s="10" t="n">
-        <f aca="false">B92*D$47</f>
-        <v>0.0174811085806451</v>
+        <f aca="false">B92*D$48</f>
+        <v>0.0167527290564515</v>
       </c>
       <c r="E92" s="10" t="n">
-        <f aca="false">B92*E$47</f>
-        <v>0.00334359202906668</v>
-      </c>
-      <c r="F92" s="18" t="n">
+        <f aca="false">B92*E$48</f>
+        <v>0.00320427569452224</v>
+      </c>
+      <c r="F92" s="17" t="n">
         <f aca="false">E92/D92</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G92" s="22" t="n">
+      <c r="G92" s="21" t="n">
         <f aca="false">E92-0.5*8*D92^2</f>
-        <v>0.00212123540023347</v>
+        <v>0.00208165997116674</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="10" t="n">
         <f aca="false">B92+0.02</f>
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="C93" s="10" t="n">
         <f aca="false">1-B93</f>
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="D93" s="10" t="n">
-        <f aca="false">B93*D$47</f>
-        <v>0.0182094881048386</v>
+        <f aca="false">B93*D$48</f>
+        <v>0.0174811085806451</v>
       </c>
       <c r="E93" s="10" t="n">
-        <f aca="false">B93*E$47</f>
-        <v>0.00348290836361113</v>
-      </c>
-      <c r="F93" s="18" t="n">
+        <f aca="false">B93*E$48</f>
+        <v>0.00334359202906668</v>
+      </c>
+      <c r="F93" s="17" t="n">
         <f aca="false">E93/D93</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G93" s="22" t="n">
+      <c r="G93" s="21" t="n">
         <f aca="false">E93-0.5*8*D93^2</f>
-        <v>0.00215656653545009</v>
+        <v>0.00212123540023347</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="10" t="n">
         <f aca="false">B93+0.02</f>
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="C94" s="10" t="n">
         <f aca="false">1-B94</f>
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="D94" s="10" t="n">
-        <f aca="false">B94*D$47</f>
-        <v>0.0189378676290322</v>
+        <f aca="false">B94*D$48</f>
+        <v>0.0182094881048386</v>
       </c>
       <c r="E94" s="10" t="n">
-        <f aca="false">B94*E$47</f>
-        <v>0.00362222469815557</v>
-      </c>
-      <c r="F94" s="18" t="n">
+        <f aca="false">B94*E$48</f>
+        <v>0.00348290836361113</v>
+      </c>
+      <c r="F94" s="17" t="n">
         <f aca="false">E94/D94</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G94" s="22" t="n">
+      <c r="G94" s="21" t="n">
         <f aca="false">E94-0.5*8*D94^2</f>
-        <v>0.00218765337681659</v>
+        <v>0.00215656653545009</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="10" t="n">
         <f aca="false">B94+0.02</f>
-        <v>0.54</v>
+        <v>0.52</v>
       </c>
       <c r="C95" s="10" t="n">
         <f aca="false">1-B95</f>
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="D95" s="10" t="n">
-        <f aca="false">B95*D$47</f>
-        <v>0.0196662471532257</v>
+        <f aca="false">B95*D$48</f>
+        <v>0.0189378676290322</v>
       </c>
       <c r="E95" s="10" t="n">
-        <f aca="false">B95*E$47</f>
-        <v>0.00376154103270002</v>
-      </c>
-      <c r="F95" s="18" t="n">
+        <f aca="false">B95*E$48</f>
+        <v>0.00362222469815557</v>
+      </c>
+      <c r="F95" s="17" t="n">
         <f aca="false">E95/D95</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G95" s="22" t="n">
+      <c r="G95" s="21" t="n">
         <f aca="false">E95-0.5*8*D95^2</f>
-        <v>0.00221449592433298</v>
+        <v>0.00218765337681659</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="10" t="n">
         <f aca="false">B95+0.02</f>
-        <v>0.56</v>
+        <v>0.54</v>
       </c>
       <c r="C96" s="10" t="n">
         <f aca="false">1-B96</f>
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="D96" s="10" t="n">
-        <f aca="false">B96*D$47</f>
-        <v>0.0203946266774192</v>
+        <f aca="false">B96*D$48</f>
+        <v>0.0196662471532257</v>
       </c>
       <c r="E96" s="10" t="n">
-        <f aca="false">B96*E$47</f>
-        <v>0.00390085736724446</v>
-      </c>
-      <c r="F96" s="18" t="n">
+        <f aca="false">B96*E$48</f>
+        <v>0.00376154103270002</v>
+      </c>
+      <c r="F96" s="17" t="n">
         <f aca="false">E96/D96</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G96" s="22" t="n">
+      <c r="G96" s="21" t="n">
         <f aca="false">E96-0.5*8*D96^2</f>
-        <v>0.00223709417799926</v>
+        <v>0.00221449592433298</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="10" t="n">
         <f aca="false">B96+0.02</f>
-        <v>0.58</v>
+        <v>0.56</v>
       </c>
       <c r="C97" s="10" t="n">
         <f aca="false">1-B97</f>
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="D97" s="10" t="n">
-        <f aca="false">B97*D$47</f>
-        <v>0.0211230062016128</v>
+        <f aca="false">B97*D$48</f>
+        <v>0.0203946266774192</v>
       </c>
       <c r="E97" s="10" t="n">
-        <f aca="false">B97*E$47</f>
-        <v>0.00404017370178891</v>
-      </c>
-      <c r="F97" s="18" t="n">
+        <f aca="false">B97*E$48</f>
+        <v>0.00390085736724446</v>
+      </c>
+      <c r="F97" s="17" t="n">
         <f aca="false">E97/D97</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G97" s="22" t="n">
+      <c r="G97" s="21" t="n">
         <f aca="false">E97-0.5*8*D97^2</f>
-        <v>0.00225544813781542</v>
+        <v>0.00223709417799926</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="10" t="n">
         <f aca="false">B97+0.02</f>
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="C98" s="10" t="n">
         <f aca="false">1-B98</f>
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="D98" s="10" t="n">
-        <f aca="false">B98*D$47</f>
-        <v>0.0218513857258063</v>
+        <f aca="false">B98*D$48</f>
+        <v>0.0211230062016128</v>
       </c>
       <c r="E98" s="10" t="n">
-        <f aca="false">B98*E$47</f>
-        <v>0.00417949003633335</v>
-      </c>
-      <c r="F98" s="18" t="n">
+        <f aca="false">B98*E$48</f>
+        <v>0.00404017370178891</v>
+      </c>
+      <c r="F98" s="17" t="n">
         <f aca="false">E98/D98</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G98" s="22" t="n">
+      <c r="G98" s="21" t="n">
         <f aca="false">E98-0.5*8*D98^2</f>
-        <v>0.00226955780378146</v>
+        <v>0.00225544813781542</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="10" t="n">
         <f aca="false">B98+0.02</f>
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="C99" s="10" t="n">
         <f aca="false">1-B99</f>
-        <v>0.38</v>
+        <v>0.4</v>
       </c>
       <c r="D99" s="10" t="n">
-        <f aca="false">B99*D$47</f>
-        <v>0.0225797652499999</v>
+        <f aca="false">B99*D$48</f>
+        <v>0.0218513857258063</v>
       </c>
       <c r="E99" s="10" t="n">
-        <f aca="false">B99*E$47</f>
-        <v>0.0043188063708778</v>
-      </c>
-      <c r="F99" s="18" t="n">
+        <f aca="false">B99*E$48</f>
+        <v>0.00417949003633335</v>
+      </c>
+      <c r="F99" s="17" t="n">
         <f aca="false">E99/D99</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G99" s="22" t="n">
+      <c r="G99" s="21" t="n">
         <f aca="false">E99-0.5*8*D99^2</f>
-        <v>0.00227942317589739</v>
+        <v>0.00226955780378146</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="10" t="n">
         <f aca="false">B99+0.02</f>
-        <v>0.64</v>
+        <v>0.62</v>
       </c>
       <c r="C100" s="10" t="n">
         <f aca="false">1-B100</f>
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="D100" s="10" t="n">
-        <f aca="false">B100*D$47</f>
-        <v>0.0233081447741934</v>
+        <f aca="false">B100*D$48</f>
+        <v>0.0225797652499999</v>
       </c>
       <c r="E100" s="10" t="n">
-        <f aca="false">B100*E$47</f>
-        <v>0.00445812270542224</v>
-      </c>
-      <c r="F100" s="18" t="n">
+        <f aca="false">B100*E$48</f>
+        <v>0.0043188063708778</v>
+      </c>
+      <c r="F100" s="17" t="n">
         <f aca="false">E100/D100</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G100" s="22" t="n">
+      <c r="G100" s="21" t="n">
         <f aca="false">E100-0.5*8*D100^2</f>
-        <v>0.0022850442541632</v>
+        <v>0.00227942317589739</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B101" s="19" t="n">
+      <c r="B101" s="10" t="n">
         <f aca="false">B100+0.02</f>
-        <v>0.66</v>
-      </c>
-      <c r="C101" s="19" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="C101" s="10" t="n">
         <f aca="false">1-B101</f>
-        <v>0.34</v>
-      </c>
-      <c r="D101" s="19" t="n">
-        <f aca="false">B101*D$47</f>
-        <v>0.024036524298387</v>
-      </c>
-      <c r="E101" s="19" t="n">
-        <f aca="false">B101*E$47</f>
-        <v>0.00459743903996669</v>
-      </c>
-      <c r="F101" s="21" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D101" s="10" t="n">
+        <f aca="false">B101*D$48</f>
+        <v>0.0233081447741934</v>
+      </c>
+      <c r="E101" s="10" t="n">
+        <f aca="false">B101*E$48</f>
+        <v>0.00445812270542224</v>
+      </c>
+      <c r="F101" s="17" t="n">
         <f aca="false">E101/D101</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G101" s="23" t="n">
+      <c r="G101" s="21" t="n">
         <f aca="false">E101-0.5*8*D101^2</f>
-        <v>0.0022864210385789</v>
+        <v>0.0022850442541632</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B102" s="10" t="n">
+      <c r="B102" s="18" t="n">
         <f aca="false">B101+0.02</f>
-        <v>0.68</v>
-      </c>
-      <c r="C102" s="10" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="C102" s="18" t="n">
         <f aca="false">1-B102</f>
-        <v>0.32</v>
-      </c>
-      <c r="D102" s="10" t="n">
-        <f aca="false">B102*D$47</f>
-        <v>0.0247649038225805</v>
-      </c>
-      <c r="E102" s="10" t="n">
-        <f aca="false">B102*E$47</f>
-        <v>0.00473675537451113</v>
-      </c>
-      <c r="F102" s="18" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="D102" s="18" t="n">
+        <f aca="false">B102*D$48</f>
+        <v>0.024036524298387</v>
+      </c>
+      <c r="E102" s="18" t="n">
+        <f aca="false">B102*E$48</f>
+        <v>0.00459743903996669</v>
+      </c>
+      <c r="F102" s="20" t="n">
         <f aca="false">E102/D102</f>
         <v>0.191268878266032</v>
       </c>
       <c r="G102" s="22" t="n">
         <f aca="false">E102-0.5*8*D102^2</f>
-        <v>0.00228355352914448</v>
+        <v>0.0022864210385789</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="10" t="n">
         <f aca="false">B102+0.02</f>
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="C103" s="10" t="n">
         <f aca="false">1-B103</f>
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="D103" s="10" t="n">
-        <f aca="false">B103*D$47</f>
-        <v>0.0254932833467741</v>
+        <f aca="false">B103*D$48</f>
+        <v>0.0247649038225805</v>
       </c>
       <c r="E103" s="10" t="n">
-        <f aca="false">B103*E$47</f>
-        <v>0.00487607170905558</v>
-      </c>
-      <c r="F103" s="18" t="n">
+        <f aca="false">B103*E$48</f>
+        <v>0.00473675537451113</v>
+      </c>
+      <c r="F103" s="17" t="n">
         <f aca="false">E103/D103</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G103" s="22" t="n">
+      <c r="G103" s="21" t="n">
         <f aca="false">E103-0.5*8*D103^2</f>
-        <v>0.00227644172585995</v>
+        <v>0.00228355352914448</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="10" t="n">
         <f aca="false">B103+0.02</f>
-        <v>0.72</v>
+        <v>0.7</v>
       </c>
       <c r="C104" s="10" t="n">
         <f aca="false">1-B104</f>
-        <v>0.28</v>
+        <v>0.3</v>
       </c>
       <c r="D104" s="10" t="n">
-        <f aca="false">B104*D$47</f>
-        <v>0.0262216628709676</v>
+        <f aca="false">B104*D$48</f>
+        <v>0.0254932833467741</v>
       </c>
       <c r="E104" s="10" t="n">
-        <f aca="false">B104*E$47</f>
-        <v>0.00501538804360002</v>
-      </c>
-      <c r="F104" s="18" t="n">
+        <f aca="false">B104*E$48</f>
+        <v>0.00487607170905558</v>
+      </c>
+      <c r="F104" s="17" t="n">
         <f aca="false">E104/D104</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G104" s="22" t="n">
+      <c r="G104" s="21" t="n">
         <f aca="false">E104-0.5*8*D104^2</f>
-        <v>0.0022650856287253</v>
+        <v>0.00227644172585995</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="10" t="n">
         <f aca="false">B104+0.02</f>
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="C105" s="10" t="n">
         <f aca="false">1-B105</f>
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="D105" s="10" t="n">
-        <f aca="false">B105*D$47</f>
-        <v>0.0269500423951611</v>
+        <f aca="false">B105*D$48</f>
+        <v>0.0262216628709676</v>
       </c>
       <c r="E105" s="10" t="n">
-        <f aca="false">B105*E$47</f>
-        <v>0.00515470437814447</v>
-      </c>
-      <c r="F105" s="18" t="n">
+        <f aca="false">B105*E$48</f>
+        <v>0.00501538804360002</v>
+      </c>
+      <c r="F105" s="17" t="n">
         <f aca="false">E105/D105</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G105" s="22" t="n">
+      <c r="G105" s="21" t="n">
         <f aca="false">E105-0.5*8*D105^2</f>
-        <v>0.00224948523774053</v>
+        <v>0.0022650856287253</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="10" t="n">
         <f aca="false">B105+0.02</f>
-        <v>0.76</v>
+        <v>0.74</v>
       </c>
       <c r="C106" s="10" t="n">
         <f aca="false">1-B106</f>
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="D106" s="10" t="n">
-        <f aca="false">B106*D$47</f>
-        <v>0.0276784219193547</v>
+        <f aca="false">B106*D$48</f>
+        <v>0.0269500423951611</v>
       </c>
       <c r="E106" s="10" t="n">
-        <f aca="false">B106*E$47</f>
-        <v>0.00529402071268891</v>
-      </c>
-      <c r="F106" s="18" t="n">
+        <f aca="false">B106*E$48</f>
+        <v>0.00515470437814447</v>
+      </c>
+      <c r="F106" s="17" t="n">
         <f aca="false">E106/D106</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G106" s="22" t="n">
+      <c r="G106" s="21" t="n">
         <f aca="false">E106-0.5*8*D106^2</f>
-        <v>0.00222964055290565</v>
+        <v>0.00224948523774053</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="10" t="n">
         <f aca="false">B106+0.02</f>
-        <v>0.78</v>
+        <v>0.76</v>
       </c>
       <c r="C107" s="10" t="n">
         <f aca="false">1-B107</f>
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="D107" s="10" t="n">
-        <f aca="false">B107*D$47</f>
-        <v>0.0284068014435482</v>
+        <f aca="false">B107*D$48</f>
+        <v>0.0276784219193547</v>
       </c>
       <c r="E107" s="10" t="n">
-        <f aca="false">B107*E$47</f>
-        <v>0.00543333704723336</v>
-      </c>
-      <c r="F107" s="18" t="n">
+        <f aca="false">B107*E$48</f>
+        <v>0.00529402071268891</v>
+      </c>
+      <c r="F107" s="17" t="n">
         <f aca="false">E107/D107</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G107" s="22" t="n">
+      <c r="G107" s="21" t="n">
         <f aca="false">E107-0.5*8*D107^2</f>
-        <v>0.00220555157422066</v>
+        <v>0.00222964055290565</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="10" t="n">
         <f aca="false">B107+0.02</f>
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="C108" s="10" t="n">
         <f aca="false">1-B108</f>
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="D108" s="10" t="n">
-        <f aca="false">B108*D$47</f>
-        <v>0.0291351809677418</v>
+        <f aca="false">B108*D$48</f>
+        <v>0.0284068014435482</v>
       </c>
       <c r="E108" s="10" t="n">
-        <f aca="false">B108*E$47</f>
-        <v>0.0055726533817778</v>
-      </c>
-      <c r="F108" s="18" t="n">
+        <f aca="false">B108*E$48</f>
+        <v>0.00543333704723336</v>
+      </c>
+      <c r="F108" s="17" t="n">
         <f aca="false">E108/D108</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G108" s="22" t="n">
+      <c r="G108" s="21" t="n">
         <f aca="false">E108-0.5*8*D108^2</f>
-        <v>0.00217721830168555</v>
+        <v>0.00220555157422066</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="10" t="n">
         <f aca="false">B108+0.02</f>
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="C109" s="10" t="n">
         <f aca="false">1-B109</f>
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="D109" s="10" t="n">
-        <f aca="false">B109*D$47</f>
-        <v>0.0298635604919353</v>
+        <f aca="false">B109*D$48</f>
+        <v>0.0291351809677418</v>
       </c>
       <c r="E109" s="10" t="n">
-        <f aca="false">B109*E$47</f>
-        <v>0.00571196971632225</v>
-      </c>
-      <c r="F109" s="18" t="n">
+        <f aca="false">B109*E$48</f>
+        <v>0.0055726533817778</v>
+      </c>
+      <c r="F109" s="17" t="n">
         <f aca="false">E109/D109</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G109" s="22" t="n">
+      <c r="G109" s="21" t="n">
         <f aca="false">E109-0.5*8*D109^2</f>
-        <v>0.00214464073530033</v>
+        <v>0.00217721830168555</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="10" t="n">
         <f aca="false">B109+0.02</f>
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="C110" s="10" t="n">
         <f aca="false">1-B110</f>
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="D110" s="10" t="n">
-        <f aca="false">B110*D$47</f>
-        <v>0.0305919400161289</v>
+        <f aca="false">B110*D$48</f>
+        <v>0.0298635604919353</v>
       </c>
       <c r="E110" s="10" t="n">
-        <f aca="false">B110*E$47</f>
-        <v>0.00585128605086669</v>
-      </c>
-      <c r="F110" s="18" t="n">
+        <f aca="false">B110*E$48</f>
+        <v>0.00571196971632225</v>
+      </c>
+      <c r="F110" s="17" t="n">
         <f aca="false">E110/D110</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G110" s="22" t="n">
+      <c r="G110" s="21" t="n">
         <f aca="false">E110-0.5*8*D110^2</f>
-        <v>0.00210781887506498</v>
+        <v>0.00214464073530033</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B111" s="10" t="n">
         <f aca="false">B110+0.02</f>
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="C111" s="10" t="n">
         <f aca="false">1-B111</f>
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="D111" s="10" t="n">
-        <f aca="false">B111*D$47</f>
-        <v>0.0313203195403224</v>
+        <f aca="false">B111*D$48</f>
+        <v>0.0305919400161289</v>
       </c>
       <c r="E111" s="10" t="n">
-        <f aca="false">B111*E$47</f>
-        <v>0.00599060238541114</v>
-      </c>
-      <c r="F111" s="18" t="n">
+        <f aca="false">B111*E$48</f>
+        <v>0.00585128605086669</v>
+      </c>
+      <c r="F111" s="17" t="n">
         <f aca="false">E111/D111</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G111" s="22" t="n">
+      <c r="G111" s="21" t="n">
         <f aca="false">E111-0.5*8*D111^2</f>
-        <v>0.00206675272097953</v>
+        <v>0.00210781887506498</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B112" s="10" t="n">
         <f aca="false">B111+0.02</f>
-        <v>0.88</v>
+        <v>0.86</v>
       </c>
       <c r="C112" s="10" t="n">
         <f aca="false">1-B112</f>
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="D112" s="10" t="n">
-        <f aca="false">B112*D$47</f>
-        <v>0.032048699064516</v>
+        <f aca="false">B112*D$48</f>
+        <v>0.0313203195403224</v>
       </c>
       <c r="E112" s="10" t="n">
-        <f aca="false">B112*E$47</f>
-        <v>0.00612991871995558</v>
-      </c>
-      <c r="F112" s="18" t="n">
+        <f aca="false">B112*E$48</f>
+        <v>0.00599060238541114</v>
+      </c>
+      <c r="F112" s="17" t="n">
         <f aca="false">E112/D112</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G112" s="22" t="n">
+      <c r="G112" s="21" t="n">
         <f aca="false">E112-0.5*8*D112^2</f>
-        <v>0.00202144227304396</v>
+        <v>0.00206675272097953</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B113" s="10" t="n">
         <f aca="false">B112+0.02</f>
-        <v>0.900000000000001</v>
+        <v>0.88</v>
       </c>
       <c r="C113" s="10" t="n">
         <f aca="false">1-B113</f>
-        <v>0.0999999999999995</v>
+        <v>0.12</v>
       </c>
       <c r="D113" s="10" t="n">
-        <f aca="false">B113*D$47</f>
-        <v>0.0327770785887095</v>
+        <f aca="false">B113*D$48</f>
+        <v>0.032048699064516</v>
       </c>
       <c r="E113" s="10" t="n">
-        <f aca="false">B113*E$47</f>
-        <v>0.00626923505450003</v>
-      </c>
-      <c r="F113" s="18" t="n">
+        <f aca="false">B113*E$48</f>
+        <v>0.00612991871995558</v>
+      </c>
+      <c r="F113" s="17" t="n">
         <f aca="false">E113/D113</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G113" s="22" t="n">
+      <c r="G113" s="21" t="n">
         <f aca="false">E113-0.5*8*D113^2</f>
-        <v>0.00197188753125827</v>
+        <v>0.00202144227304396</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B114" s="10" t="n">
         <f aca="false">B113+0.02</f>
-        <v>0.920000000000001</v>
+        <v>0.900000000000001</v>
       </c>
       <c r="C114" s="10" t="n">
         <f aca="false">1-B114</f>
-        <v>0.0799999999999995</v>
+        <v>0.0999999999999995</v>
       </c>
       <c r="D114" s="10" t="n">
-        <f aca="false">B114*D$47</f>
-        <v>0.0335054581129031</v>
+        <f aca="false">B114*D$48</f>
+        <v>0.0327770785887095</v>
       </c>
       <c r="E114" s="10" t="n">
-        <f aca="false">B114*E$47</f>
-        <v>0.00640855138904447</v>
-      </c>
-      <c r="F114" s="18" t="n">
+        <f aca="false">B114*E$48</f>
+        <v>0.00626923505450003</v>
+      </c>
+      <c r="F114" s="17" t="n">
         <f aca="false">E114/D114</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G114" s="22" t="n">
+      <c r="G114" s="21" t="n">
         <f aca="false">E114-0.5*8*D114^2</f>
-        <v>0.00191808849562247</v>
+        <v>0.00197188753125827</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B115" s="10" t="n">
         <f aca="false">B114+0.02</f>
-        <v>0.940000000000001</v>
+        <v>0.920000000000001</v>
       </c>
       <c r="C115" s="10" t="n">
         <f aca="false">1-B115</f>
-        <v>0.0599999999999995</v>
+        <v>0.0799999999999995</v>
       </c>
       <c r="D115" s="10" t="n">
-        <f aca="false">B115*D$47</f>
-        <v>0.0342338376370966</v>
+        <f aca="false">B115*D$48</f>
+        <v>0.0335054581129031</v>
       </c>
       <c r="E115" s="10" t="n">
-        <f aca="false">B115*E$47</f>
-        <v>0.00654786772358892</v>
-      </c>
-      <c r="F115" s="18" t="n">
+        <f aca="false">B115*E$48</f>
+        <v>0.00640855138904447</v>
+      </c>
+      <c r="F115" s="17" t="n">
         <f aca="false">E115/D115</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G115" s="22" t="n">
+      <c r="G115" s="21" t="n">
         <f aca="false">E115-0.5*8*D115^2</f>
-        <v>0.00186004516613655</v>
+        <v>0.00191808849562247</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="10" t="n">
         <f aca="false">B115+0.02</f>
-        <v>0.960000000000001</v>
+        <v>0.940000000000001</v>
       </c>
       <c r="C116" s="10" t="n">
         <f aca="false">1-B116</f>
-        <v>0.0399999999999995</v>
+        <v>0.0599999999999995</v>
       </c>
       <c r="D116" s="10" t="n">
-        <f aca="false">B116*D$47</f>
-        <v>0.0349622171612901</v>
+        <f aca="false">B116*D$48</f>
+        <v>0.0342338376370966</v>
       </c>
       <c r="E116" s="10" t="n">
-        <f aca="false">B116*E$47</f>
-        <v>0.00668718405813336</v>
-      </c>
-      <c r="F116" s="18" t="n">
+        <f aca="false">B116*E$48</f>
+        <v>0.00654786772358892</v>
+      </c>
+      <c r="F116" s="17" t="n">
         <f aca="false">E116/D116</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G116" s="22" t="n">
+      <c r="G116" s="21" t="n">
         <f aca="false">E116-0.5*8*D116^2</f>
-        <v>0.00179775754280052</v>
+        <v>0.00186004516613655</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="10" t="n">
         <f aca="false">B116+0.02</f>
-        <v>0.980000000000001</v>
+        <v>0.960000000000001</v>
       </c>
       <c r="C117" s="10" t="n">
         <f aca="false">1-B117</f>
-        <v>0.0199999999999995</v>
+        <v>0.0399999999999995</v>
       </c>
       <c r="D117" s="10" t="n">
-        <f aca="false">B117*D$47</f>
-        <v>0.0356905966854837</v>
+        <f aca="false">B117*D$48</f>
+        <v>0.0349622171612901</v>
       </c>
       <c r="E117" s="10" t="n">
-        <f aca="false">B117*E$47</f>
-        <v>0.00682650039267781</v>
-      </c>
-      <c r="F117" s="18" t="n">
+        <f aca="false">B117*E$48</f>
+        <v>0.00668718405813336</v>
+      </c>
+      <c r="F117" s="17" t="n">
         <f aca="false">E117/D117</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G117" s="22" t="n">
+      <c r="G117" s="21" t="n">
         <f aca="false">E117-0.5*8*D117^2</f>
-        <v>0.00173122562561437</v>
+        <v>0.00179775754280052</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B118" s="10" t="n">
         <f aca="false">B117+0.02</f>
-        <v>1</v>
+        <v>0.980000000000001</v>
       </c>
       <c r="C118" s="10" t="n">
         <f aca="false">1-B118</f>
-        <v>0</v>
+        <v>0.0199999999999995</v>
       </c>
       <c r="D118" s="10" t="n">
-        <f aca="false">B118*D$47</f>
-        <v>0.0364189762096772</v>
+        <f aca="false">B118*D$48</f>
+        <v>0.0356905966854837</v>
       </c>
       <c r="E118" s="10" t="n">
-        <f aca="false">B118*E$47</f>
-        <v>0.00696581672722225</v>
-      </c>
-      <c r="F118" s="18" t="n">
+        <f aca="false">B118*E$48</f>
+        <v>0.00682650039267781</v>
+      </c>
+      <c r="F118" s="17" t="n">
         <f aca="false">E118/D118</f>
         <v>0.191268878266032</v>
       </c>
-      <c r="G118" s="22" t="n">
+      <c r="G118" s="21" t="n">
         <f aca="false">E118-0.5*8*D118^2</f>
+        <v>0.00173122562561437</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B119" s="10" t="n">
+        <f aca="false">B118+0.02</f>
+        <v>1</v>
+      </c>
+      <c r="C119" s="10" t="n">
+        <f aca="false">1-B119</f>
+        <v>0</v>
+      </c>
+      <c r="D119" s="10" t="n">
+        <f aca="false">B119*D$48</f>
+        <v>0.0364189762096772</v>
+      </c>
+      <c r="E119" s="10" t="n">
+        <f aca="false">B119*E$48</f>
+        <v>0.00696581672722225</v>
+      </c>
+      <c r="F119" s="17" t="n">
+        <f aca="false">E119/D119</f>
+        <v>0.191268878266032</v>
+      </c>
+      <c r="G119" s="21" t="n">
+        <f aca="false">E119-0.5*8*D119^2</f>
         <v>0.00166044941457811</v>
       </c>
     </row>
@@ -27974,7 +28000,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
     </row>
@@ -27986,7 +28012,7 @@
         <v>6</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>5</v>
@@ -28014,7 +28040,7 @@
         <f aca="false">B4^2</f>
         <v>0.00154601681310119</v>
       </c>
-      <c r="G3" s="24" t="n">
+      <c r="G3" s="23" t="n">
         <f aca="false">B6</f>
         <v>0.000578833690489693</v>
       </c>
@@ -28034,7 +28060,7 @@
       <c r="E4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="23" t="n">
         <f aca="false">B6</f>
         <v>0.000578833690489693</v>
       </c>
@@ -28045,33 +28071,33 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B5" s="14" t="n">
         <f aca="false">CORREL('Excess returns'!C3:C242,'Excess returns'!D3:D242)</f>
         <v>0.241426381441205</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="B6" s="14" t="n">
         <f aca="false">B5*B4*C4</f>
         <v>0.000578833690489693</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>24</v>
+      <c r="A8" s="24" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="14" t="s">
+      <c r="A10" s="12" t="s">
         <v>26</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28090,7 +28116,7 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.72</v>
@@ -28100,11 +28126,11 @@
         <v>0.28</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="26" t="n">
+        <v>29</v>
+      </c>
+      <c r="F12" s="25" t="n">
         <f aca="false" t="array" ref="F12:G12">TRANSPOSE( MMULT( MINVERSE( F3:G4 ) , TRANSPOSE(B3:C3) ))</f>
-        <v>3.78224432984199</v>
+        <v>3.782244329842</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>1.46976687866939</v>
@@ -28112,29 +28138,29 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E13" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F13" s="1" t="n">
         <f aca="false">F12/(F12+G12)</f>
-        <v>0.720151610436875</v>
+        <v>0.720151610436876</v>
       </c>
       <c r="G13" s="1" t="n">
         <f aca="false">G12/(F12+G12)</f>
-        <v>0.279848389563125</v>
+        <v>0.279848389563124</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="22" t="n">
+      <c r="B14" s="21" t="n">
         <f aca="false">B12*B3+C12*C3</f>
         <v>0.00696581672722225</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F14" s="21" t="n">
         <f aca="false">F13*B3 + G13*C3</f>
         <v>0.00696567180236408</v>
       </c>
@@ -28143,36 +28169,36 @@
       <c r="A15" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B15" s="21" t="n">
         <f aca="false">SQRT(B12^2*B4^2 + C12^2*C4^2 + 2*B12*C12*B6)</f>
         <v>0.0364189762096772</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F15" s="22" t="n">
+      <c r="F15" s="21" t="n">
         <f aca="false">SQRT( F13^2*B4^2 + G13^2*C4^2 + 2*F13*G13*B6)</f>
         <v>0.0364182172194484</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="22" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="21" t="n">
         <f aca="false">B14/B15</f>
         <v>0.191268878266032</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F16" s="22" t="n">
+        <v>14</v>
+      </c>
+      <c r="F16" s="21" t="n">
         <f aca="false">F14/F15</f>
         <v>0.191268885030545</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="24" t="s">
         <v>31</v>
       </c>
     </row>
@@ -28185,10 +28211,10 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="E22" s="14" t="s">
+      <c r="A22" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="12" t="s">
         <v>33</v>
       </c>
     </row>
@@ -28204,7 +28230,7 @@
       </c>
       <c r="F23" s="10" t="n">
         <f aca="false">F14/(B20*F15^2)</f>
-        <v>0.656501401063923</v>
+        <v>0.656501401063922</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28220,7 +28246,7 @@
       </c>
       <c r="F24" s="10" t="n">
         <f aca="false">F23*F14</f>
-        <v>0.00457297329760348</v>
+        <v>0.00457297329760347</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28243,28 +28269,28 @@
       <c r="A26" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="22" t="n">
+      <c r="B26" s="21" t="n">
         <f aca="false">B24 - 0.5*B20*B25^2</f>
         <v>0.0022864210385789</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F26" s="22" t="n">
+      <c r="F26" s="21" t="n">
         <f aca="false">F24 - 0.5*B20*F25^2</f>
         <v>0.00228648664880174</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="24" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25"/>
+      <c r="A29" s="24"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="27" t="s">
+      <c r="A30" s="26" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>